<commit_message>
Actualizacion de documentos y avances de BI Copilot
</commit_message>
<xml_diff>
--- a/seccion/grupo5/Fase 2/Evidencias Grupales/PLANILLA DE EVALUACION AVANCE FASE 2.xlsx
+++ b/seccion/grupo5/Fase 2/Evidencias Grupales/PLANILLA DE EVALUACION AVANCE FASE 2.xlsx
@@ -11,40 +11,40 @@
     <sheet state="hidden" name="RELEVANCIA-PUNTAJE" sheetId="6" r:id="rId10"/>
   </sheets>
   <definedNames>
+    <definedName name="MR_NL">'RELEVANCIA-PUNTAJE'!$E$3</definedName>
+    <definedName name="TL">'RELEVANCIA-PUNTAJE'!$B$2</definedName>
+    <definedName name="ML">'RELEVANCIA-PUNTAJE'!$D$2</definedName>
+    <definedName name="CL">'RELEVANCIA-PUNTAJE'!$B$2</definedName>
+    <definedName name="PR_ML">'RELEVANCIA-PUNTAJE'!$D$5</definedName>
     <definedName name="MR_L">'RELEVANCIA-PUNTAJE'!$C$3</definedName>
+    <definedName name="RE_ML">'RELEVANCIA-PUNTAJE'!$D$4</definedName>
+    <definedName name="PR_NL">'RELEVANCIA-PUNTAJE'!$E$5</definedName>
+    <definedName name="MR_CL">'RELEVANCIA-PUNTAJE'!$B$3</definedName>
+    <definedName name="RE_NL">'RELEVANCIA-PUNTAJE'!$E$4</definedName>
     <definedName name="RE_TL">'RELEVANCIA-PUNTAJE'!$B$4</definedName>
+    <definedName name="NL">'RELEVANCIA-PUNTAJE'!$E$2</definedName>
+    <definedName name="PR_TL">'RELEVANCIA-PUNTAJE'!$B$5</definedName>
+    <definedName name="MR_ML">'RELEVANCIA-PUNTAJE'!$D$3</definedName>
+    <definedName name="PR">'RELEVANCIA-PUNTAJE'!$A$5</definedName>
+    <definedName name="MR_TL">'RELEVANCIA-PUNTAJE'!$B$3</definedName>
     <definedName name="RE">'RELEVANCIA-PUNTAJE'!$A$4</definedName>
-    <definedName name="PR_ML">'RELEVANCIA-PUNTAJE'!$D$5</definedName>
-    <definedName name="CL">'RELEVANCIA-PUNTAJE'!$B$2</definedName>
-    <definedName name="MR_ML">'RELEVANCIA-PUNTAJE'!$D$3</definedName>
     <definedName name="MR">'RELEVANCIA-PUNTAJE'!$A$3</definedName>
-    <definedName name="PR_TL">'RELEVANCIA-PUNTAJE'!$B$5</definedName>
-    <definedName name="ML">'RELEVANCIA-PUNTAJE'!$D$2</definedName>
-    <definedName name="PR">'RELEVANCIA-PUNTAJE'!$A$5</definedName>
-    <definedName name="RE_NL">'RELEVANCIA-PUNTAJE'!$E$4</definedName>
-    <definedName name="PR_NL">'RELEVANCIA-PUNTAJE'!$E$5</definedName>
-    <definedName name="MR_NL">'RELEVANCIA-PUNTAJE'!$E$3</definedName>
-    <definedName name="NL">'RELEVANCIA-PUNTAJE'!$E$2</definedName>
     <definedName name="L">'RELEVANCIA-PUNTAJE'!$C$2</definedName>
-    <definedName name="TL">'RELEVANCIA-PUNTAJE'!$B$2</definedName>
-    <definedName name="MR_TL">'RELEVANCIA-PUNTAJE'!$B$3</definedName>
-    <definedName name="RE_ML">'RELEVANCIA-PUNTAJE'!$D$4</definedName>
-    <definedName name="MR_CL">'RELEVANCIA-PUNTAJE'!$B$3</definedName>
   </definedNames>
   <calcPr/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="63">
-  <si>
-    <t>PUNTOS</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="66">
   <si>
     <t>Puntaje</t>
   </si>
   <si>
     <t>Indicador de Evaluación</t>
+  </si>
+  <si>
+    <t>PUNTOS</t>
   </si>
   <si>
     <t>Nota</t>
@@ -53,16 +53,19 @@
     <t>NOTA</t>
   </si>
   <si>
+    <t>Categorías de Respuesta</t>
+  </si>
+  <si>
     <t>INTEGRANTES</t>
   </si>
   <si>
     <t>GRUPAL</t>
   </si>
   <si>
-    <t>Categorías de Respuesta</t>
+    <t>Ponderación del Indicador de Evaluación</t>
   </si>
   <si>
-    <t>Ponderación del Indicador de Evaluación</t>
+    <t>CARRASCO FIGUEROA IGNACIO ANTONIO</t>
   </si>
   <si>
     <r>
@@ -111,22 +114,22 @@
     <t>No logrado</t>
   </si>
   <si>
+    <t>NAVARRO CONTRERAS VALENTIN ANDRES</t>
+  </si>
+  <si>
     <t xml:space="preserve">1. Propone ajustes al Proyecto APT considerando dificultades, facilitadores y retroalimentación. </t>
   </si>
   <si>
-    <t>Señala los ajustes que realizó o realizará y los justifica considerando las dificultades, facilitadores y retroalimentación del docente.</t>
+    <t>PINERA CAVIERES FELIPE ALEXIS</t>
   </si>
   <si>
-    <t>Nivel de Logro</t>
+    <t>Señala los ajustes que realizó o realizará y los justifica considerando las dificultades, facilitadores y retroalimentación del docente.</t>
   </si>
   <si>
     <t>Señala algunos de los ajustes que realizó o realizará y los justifica considerando las dificultades, facilitadores o retroalimentación del docente.</t>
   </si>
   <si>
     <t>Señala los ajustes que realizó o realizará, pero no los justifica.</t>
-  </si>
-  <si>
-    <t>NIVELES DE LOGRO Y PUNTAJES</t>
   </si>
   <si>
     <t>No incluye ajustes ni justifica por qué mantiene su plan inicial.</t>
@@ -138,13 +141,7 @@
     <t xml:space="preserve">Aplica la metodología definida por el equipo de acuerdo a los estándares de la disciplina, alcanzando los objetivos propuestos para el avance del proyecto. </t>
   </si>
   <si>
-    <t>Aspectos a Evaluar</t>
-  </si>
-  <si>
     <t xml:space="preserve">Aplica la metodología definida de acuerdo a los estándares de la disciplina, pero no se observa el cumplimiento de objetivos propuestos para el avance del proyecto. </t>
-  </si>
-  <si>
-    <t>Completamente logrado</t>
   </si>
   <si>
     <t xml:space="preserve">Aplica la metodología definida cumpliendo parcialmente con los estándares de la disciplina y con los objetivos propuestos para el avance del proyecto. </t>
@@ -153,13 +150,7 @@
     <t xml:space="preserve">Aplica la metodología definida sin cumplir los estándares de la disciplina ni los objetivos propuestos para el avance del proyecto. </t>
   </si>
   <si>
-    <t>Logrado</t>
-  </si>
-  <si>
     <t>3. Genera evidencias que dan cuenta del avance del Proyecto APT en relación a documentación, programación y almacenamiento de datos , de acuerdo a lo planificado por el equipo y que cumpla con estándares de desarrollo de la industria</t>
-  </si>
-  <si>
-    <t>Logro Incipiente</t>
   </si>
   <si>
     <t>Presenta evidencias de avance que cumplen con lo planificado por el equipo en relación a documentación, programación y almacenamiento de datos, entregando evidencias que cumplan con estándares de desarrollo que actualmente se encuentran presentes en la industria</t>
@@ -234,6 +225,9 @@
     <t>No generan evidencias dentro del repositorio  del proyecto del aporte de cada uno de los integrantes del equipo por lo que no se permite identificar la equidad en el trabajo y la participación de cada estudiante</t>
   </si>
   <si>
+    <t>Nivel de Logro</t>
+  </si>
+  <si>
     <t>8. Demuestra un trabajo en equipo en donde todos los miembros del equipo expresan con fluidez el conocimiento del tema expuesto y  participan de las actividades planificadas en el proyecto</t>
   </si>
   <si>
@@ -246,7 +240,22 @@
     <t>Demuestra de manera deficiente el trabajo en equipo en donde los integrantes expresan con poca fluidez y de manera imparcial el conocimiento del tema expuesto y no todos sus miembros participan de manera equitativa de las actividades planificadas en el proyecto</t>
   </si>
   <si>
+    <t>NIVELES DE LOGRO Y PUNTAJES</t>
+  </si>
+  <si>
     <t xml:space="preserve">No demuestran un trabajo en equipo, evidenciando en su presentación la nula colaboración de alguno de sus integrantes. </t>
+  </si>
+  <si>
+    <t>Aspectos a Evaluar</t>
+  </si>
+  <si>
+    <t>Completamente logrado</t>
+  </si>
+  <si>
+    <t>Logrado</t>
+  </si>
+  <si>
+    <t>Logro Incipiente</t>
   </si>
   <si>
     <t>Relevancia</t>
@@ -268,7 +277,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="16">
     <font>
       <sz val="11.0"/>
       <color rgb="FF000000"/>
@@ -278,15 +287,8 @@
     <font>
       <color theme="1"/>
       <name val="Calibri"/>
-      <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11.0"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11.0"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
@@ -297,11 +299,33 @@
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11.0"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+    </font>
     <font/>
+    <font>
+      <sz val="11.0"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+    </font>
     <font>
       <b/>
       <sz val="11.0"/>
       <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10.0"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10.0"/>
+      <color rgb="FF3B3838"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -311,7 +335,7 @@
     </font>
     <font>
       <sz val="10.0"/>
-      <color rgb="FF000000"/>
+      <color theme="1"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -327,19 +351,8 @@
       <name val="Calibri"/>
     </font>
     <font>
-      <b/>
-      <sz val="10.0"/>
-      <color rgb="FF3B3838"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
       <sz val="9.0"/>
       <color rgb="FF000000"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10.0"/>
-      <color theme="1"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -386,7 +399,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="28">
+  <borders count="27">
     <border/>
     <border>
       <left style="thin">
@@ -412,17 +425,6 @@
       <top style="medium">
         <color rgb="FF7F7F7F"/>
       </top>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
     </border>
     <border>
       <left style="medium">
@@ -477,17 +479,27 @@
       <right style="medium">
         <color rgb="FF7F7F7F"/>
       </right>
-      <bottom/>
+      <bottom style="medium">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
     </border>
     <border>
-      <left style="medium">
-        <color rgb="FF7F7F7F"/>
-      </left>
       <right style="medium">
         <color rgb="FF7F7F7F"/>
       </right>
       <bottom style="medium">
         <color rgb="FF7F7F7F"/>
+      </bottom>
+    </border>
+    <border>
+      <right style="medium">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
       </bottom>
     </border>
     <border>
@@ -502,11 +514,14 @@
       </top>
     </border>
     <border>
-      <right style="medium">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <bottom style="medium">
-        <color rgb="FF7F7F7F"/>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
       </bottom>
     </border>
     <border>
@@ -555,17 +570,6 @@
       <right style="thin">
         <color rgb="FF000000"/>
       </right>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-    </border>
-    <border>
-      <right style="medium">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF7F7F7F"/>
-      </top>
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
@@ -668,134 +672,136 @@
     <xf borderId="1" fillId="2" fontId="2" numFmtId="9" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
+    <xf borderId="2" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyFont="1" applyNumberFormat="1"/>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="2" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="3" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
+    <xf borderId="4" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left"/>
+    <xf borderId="5" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="1" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment vertical="bottom"/>
     </xf>
-    <xf borderId="4" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="5" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="6" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="7" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="2" fillId="3" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="2" fillId="3" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="2" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="8" fillId="3" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="7" fillId="3" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="8" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="7" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="9" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="8" fillId="3" fontId="4" numFmtId="9" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="7" fillId="3" fontId="3" numFmtId="9" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="10" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="11" fillId="4" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" textRotation="255" vertical="center"/>
-    </xf>
+    <xf borderId="8" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="1" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="5" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="9" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="10" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="11" fillId="4" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" textRotation="255" vertical="center"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="5" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="11" fillId="5" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="9" fillId="0" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="11" fillId="5" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="3" fillId="5" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="10" fillId="0" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="12" fillId="5" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="12" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="13" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="14" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="15" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="16" fillId="5" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="16" fillId="5" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf borderId="17" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="1" fillId="0" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="0" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="18" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf borderId="14" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf borderId="14" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="18" fillId="5" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf borderId="19" fillId="5" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="12" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf borderId="20" fillId="5" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="18" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf borderId="21" fillId="5" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="19" fillId="5" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="22" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="23" fillId="5" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="24" fillId="5" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="25" fillId="5" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="22" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="20" fillId="5" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="21" fillId="5" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="22" fillId="5" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="23" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="24" fillId="5" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="25" fillId="5" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="26" fillId="5" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="23" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="26" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="27" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="17" fillId="0" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="17" fillId="0" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="right" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="11" fillId="0" fontId="14" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="11" fillId="0" fontId="15" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="1" fillId="6" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
-    <xf borderId="3" fillId="0" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="12" fillId="0" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="right" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="14" numFmtId="164" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="1" fillId="0" fontId="15" numFmtId="164" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="right" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="14" numFmtId="164" xfId="0" applyFont="1" applyNumberFormat="1"/>
-    <xf borderId="0" fillId="0" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="15" numFmtId="164" xfId="0" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="0" fillId="0" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1062,442 +1068,448 @@
       </c>
     </row>
     <row r="3">
-      <c r="B3" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3" s="6" t="s">
+      <c r="B3" s="5" t="s">
         <v>6</v>
       </c>
+      <c r="C3" s="7" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="7">
+      <c r="A4" s="9">
         <v>1.0</v>
       </c>
-      <c r="B4" s="8"/>
+      <c r="B4" s="11" t="s">
+        <v>9</v>
+      </c>
       <c r="C4" s="14">
         <f>EVALUACION2!$C$22</f>
-        <v>7</v>
-      </c>
-      <c r="G4" s="3"/>
+        <v>5.8</v>
+      </c>
+      <c r="G4" s="4"/>
     </row>
     <row r="5">
-      <c r="A5" s="7">
+      <c r="A5" s="9">
         <v>2.0</v>
       </c>
-      <c r="B5" s="8"/>
+      <c r="B5" s="11" t="s">
+        <v>14</v>
+      </c>
       <c r="C5" s="14">
         <f>EVALUACION2!$C$22</f>
-        <v>7</v>
-      </c>
-      <c r="G5" s="3"/>
+        <v>5.8</v>
+      </c>
+      <c r="G5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="7">
+      <c r="A6" s="9">
         <v>3.0</v>
       </c>
-      <c r="B6" s="8"/>
+      <c r="B6" s="11" t="s">
+        <v>16</v>
+      </c>
       <c r="C6" s="14">
         <f>EVALUACION2!$C$22</f>
+        <v>5.8</v>
+      </c>
+      <c r="G6" s="4"/>
+    </row>
+    <row r="11" outlineLevel="1">
+      <c r="A11" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="G6" s="3"/>
-    </row>
-    <row r="11" outlineLevel="1">
-      <c r="A11" s="20" t="s">
-        <v>6</v>
-      </c>
-      <c r="B11" s="22"/>
-      <c r="C11" s="23" t="s">
-        <v>15</v>
-      </c>
-      <c r="D11" s="24" t="s">
-        <v>18</v>
-      </c>
-      <c r="E11" s="26"/>
-      <c r="F11" s="26"/>
-      <c r="G11" s="26"/>
-      <c r="H11" s="26"/>
-      <c r="I11" s="26"/>
-      <c r="J11" s="26"/>
-      <c r="K11" s="27"/>
+      <c r="B11" s="24"/>
+      <c r="C11" s="26" t="s">
+        <v>51</v>
+      </c>
+      <c r="D11" s="28" t="s">
+        <v>56</v>
+      </c>
+      <c r="E11" s="29"/>
+      <c r="F11" s="29"/>
+      <c r="G11" s="29"/>
+      <c r="H11" s="29"/>
+      <c r="I11" s="29"/>
+      <c r="J11" s="29"/>
+      <c r="K11" s="30"/>
     </row>
     <row r="12" outlineLevel="1">
-      <c r="A12" s="28"/>
-      <c r="B12" s="29" t="s">
-        <v>22</v>
-      </c>
-      <c r="C12" s="30"/>
-      <c r="D12" s="24" t="s">
-        <v>24</v>
-      </c>
-      <c r="E12" s="27"/>
-      <c r="F12" s="24" t="s">
-        <v>27</v>
-      </c>
-      <c r="G12" s="27"/>
-      <c r="H12" s="24" t="s">
-        <v>29</v>
-      </c>
-      <c r="I12" s="27"/>
-      <c r="J12" s="24" t="s">
-        <v>12</v>
-      </c>
-      <c r="K12" s="27"/>
+      <c r="A12" s="31"/>
+      <c r="B12" s="32" t="s">
+        <v>58</v>
+      </c>
+      <c r="C12" s="33"/>
+      <c r="D12" s="28" t="s">
+        <v>59</v>
+      </c>
+      <c r="E12" s="30"/>
+      <c r="F12" s="28" t="s">
+        <v>60</v>
+      </c>
+      <c r="G12" s="30"/>
+      <c r="H12" s="28" t="s">
+        <v>61</v>
+      </c>
+      <c r="I12" s="30"/>
+      <c r="J12" s="28" t="s">
+        <v>13</v>
+      </c>
+      <c r="K12" s="30"/>
     </row>
     <row r="13" outlineLevel="1">
-      <c r="A13" s="28"/>
-      <c r="B13" s="31" t="str">
+      <c r="A13" s="31"/>
+      <c r="B13" s="34" t="str">
         <f>RUBRICA!A4</f>
         <v>1. Propone ajustes al Proyecto APT considerando dificultades, facilitadores y retroalimentación. </v>
       </c>
-      <c r="C13" s="33" t="s">
-        <v>24</v>
-      </c>
-      <c r="D13" s="35" t="str">
+      <c r="C13" s="35" t="s">
+        <v>59</v>
+      </c>
+      <c r="D13" s="36" t="str">
         <f>IF($C13=CL,"X","")</f>
         <v>X</v>
       </c>
-      <c r="E13" s="35">
+      <c r="E13" s="36">
         <f t="shared" ref="E13:E14" si="1">IF(D13="X",100*0.1,"")</f>
         <v>10</v>
       </c>
-      <c r="F13" s="35" t="str">
+      <c r="F13" s="36" t="str">
         <f>IF($C13=L,"X","")</f>
         <v/>
       </c>
-      <c r="G13" s="35" t="str">
+      <c r="G13" s="36" t="str">
         <f t="shared" ref="G13:G14" si="2">IF(F13="X",60*0.1,"")</f>
         <v/>
       </c>
-      <c r="H13" s="35" t="str">
+      <c r="H13" s="36" t="str">
         <f>IF($C13=ML,"X","")</f>
         <v/>
       </c>
-      <c r="I13" s="35" t="str">
+      <c r="I13" s="36" t="str">
         <f t="shared" ref="I13:I14" si="3">IF(H13="X",30*0.1,"")</f>
         <v/>
       </c>
-      <c r="J13" s="35" t="str">
+      <c r="J13" s="36" t="str">
         <f>IF($C13=NL,"X","")</f>
         <v/>
       </c>
-      <c r="K13" s="35" t="str">
+      <c r="K13" s="36" t="str">
         <f t="shared" ref="K13:K20" si="4">IF($J13="X",0,"")</f>
         <v/>
       </c>
     </row>
     <row r="14" ht="26.25" customHeight="1" outlineLevel="1">
-      <c r="A14" s="28"/>
-      <c r="B14" s="31" t="str">
+      <c r="A14" s="31"/>
+      <c r="B14" s="34" t="str">
         <f>RUBRICA!A5</f>
         <v>2. Aplica una metodología que permite el logro de los objetivos propuestos, de acuerdo a los estándares de la disciplina.</v>
       </c>
-      <c r="C14" s="33" t="s">
-        <v>24</v>
-      </c>
-      <c r="D14" s="35" t="str">
+      <c r="C14" s="37" t="s">
+        <v>59</v>
+      </c>
+      <c r="D14" s="36" t="str">
         <f>IF($C14=CL,"X","")</f>
         <v>X</v>
       </c>
-      <c r="E14" s="35">
+      <c r="E14" s="36">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="F14" s="35" t="str">
+      <c r="F14" s="36" t="str">
         <f>IF($C14=L,"X","")</f>
         <v/>
       </c>
-      <c r="G14" s="35" t="str">
+      <c r="G14" s="36" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="H14" s="35" t="str">
+      <c r="H14" s="36" t="str">
         <f>IF($C14=ML,"X","")</f>
         <v/>
       </c>
-      <c r="I14" s="35" t="str">
+      <c r="I14" s="36" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="J14" s="35" t="str">
+      <c r="J14" s="36" t="str">
         <f>IF($C14=NL,"X","")</f>
         <v/>
       </c>
-      <c r="K14" s="35" t="str">
+      <c r="K14" s="36" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
     </row>
     <row r="15" outlineLevel="1">
-      <c r="A15" s="28"/>
-      <c r="B15" s="31" t="str">
+      <c r="A15" s="31"/>
+      <c r="B15" s="34" t="str">
         <f>RUBRICA!A6</f>
         <v>3. Genera evidencias que dan cuenta del avance del Proyecto APT en relación a documentación, programación y almacenamiento de datos , de acuerdo a lo planificado por el equipo y que cumpla con estándares de desarrollo de la industria</v>
       </c>
-      <c r="C15" s="33" t="s">
-        <v>24</v>
-      </c>
-      <c r="D15" s="35" t="str">
+      <c r="C15" s="37" t="s">
+        <v>59</v>
+      </c>
+      <c r="D15" s="36" t="str">
         <f>IF($C15=CL,"X","")</f>
         <v>X</v>
       </c>
-      <c r="E15" s="35">
+      <c r="E15" s="36">
         <f>IF(D15="X",100*0.25,"")</f>
         <v>25</v>
       </c>
-      <c r="F15" s="35" t="str">
+      <c r="F15" s="36" t="str">
         <f>IF($C15=L,"X","")</f>
         <v/>
       </c>
-      <c r="G15" s="35" t="str">
+      <c r="G15" s="36" t="str">
         <f>IF(F15="X",60*0.25,"")</f>
         <v/>
       </c>
-      <c r="H15" s="35" t="str">
+      <c r="H15" s="36" t="str">
         <f>IF($C15=ML,"X","")</f>
         <v/>
       </c>
-      <c r="I15" s="35" t="str">
+      <c r="I15" s="36" t="str">
         <f>IF(H15="X",30*0.25,"")</f>
         <v/>
       </c>
-      <c r="J15" s="35" t="str">
+      <c r="J15" s="36" t="str">
         <f>IF($C15=NL,"X","")</f>
         <v/>
       </c>
-      <c r="K15" s="35" t="str">
+      <c r="K15" s="36" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
     </row>
     <row r="16" outlineLevel="1">
-      <c r="A16" s="28"/>
-      <c r="B16" s="31" t="str">
+      <c r="A16" s="31"/>
+      <c r="B16" s="34" t="str">
         <f>RUBRICA!A7</f>
         <v>4. Utiliza de manera precisa el lenguaje técnico en los entregables de acuerdo con lo requerido por la disciplina.</v>
       </c>
-      <c r="C16" s="33" t="s">
-        <v>24</v>
-      </c>
-      <c r="D16" s="35" t="str">
+      <c r="C16" s="37" t="s">
+        <v>59</v>
+      </c>
+      <c r="D16" s="36" t="str">
         <f>IF($C16=CL,"X","")</f>
         <v>X</v>
       </c>
-      <c r="E16" s="35">
+      <c r="E16" s="36">
         <f t="shared" ref="E16:E17" si="5">IF(D16="X",100*0.05,"")</f>
         <v>5</v>
       </c>
-      <c r="F16" s="35" t="str">
+      <c r="F16" s="36" t="str">
         <f>IF($C16=L,"X","")</f>
         <v/>
       </c>
-      <c r="G16" s="35" t="str">
+      <c r="G16" s="36" t="str">
         <f t="shared" ref="G16:G17" si="6">IF(F16="X",60*0.05,"")</f>
         <v/>
       </c>
-      <c r="H16" s="35" t="str">
+      <c r="H16" s="36" t="str">
         <f>IF($C16=ML,"X","")</f>
         <v/>
       </c>
-      <c r="I16" s="35" t="str">
+      <c r="I16" s="36" t="str">
         <f t="shared" ref="I16:I17" si="7">IF(H16="X",30*0.05,"")</f>
         <v/>
       </c>
-      <c r="J16" s="35" t="str">
+      <c r="J16" s="36" t="str">
         <f>IF($C16=NL,"X","")</f>
         <v/>
       </c>
-      <c r="K16" s="35" t="str">
+      <c r="K16" s="36" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
     </row>
     <row r="17" outlineLevel="1">
-      <c r="A17" s="28"/>
-      <c r="B17" s="31" t="str">
+      <c r="A17" s="31"/>
+      <c r="B17" s="34" t="str">
         <f>RUBRICA!A8</f>
         <v>5. Utiliza reglas de redacción, ortografía (literal, puntual, acentual) y las normas para citas y referencias. </v>
       </c>
-      <c r="C17" s="33" t="s">
-        <v>24</v>
-      </c>
-      <c r="D17" s="35" t="str">
+      <c r="C17" s="35" t="s">
+        <v>60</v>
+      </c>
+      <c r="D17" s="36" t="str">
         <f>IF($C17=CL,"X","")</f>
+        <v/>
+      </c>
+      <c r="E17" s="36" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+      <c r="F17" s="36" t="str">
+        <f>IF($C17=L,"X","")</f>
         <v>X</v>
       </c>
-      <c r="E17" s="35">
-        <f t="shared" si="5"/>
-        <v>5</v>
-      </c>
-      <c r="F17" s="35" t="str">
-        <f>IF($C17=L,"X","")</f>
-        <v/>
-      </c>
-      <c r="G17" s="35" t="str">
+      <c r="G17" s="36">
         <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="H17" s="35" t="str">
+        <v>3</v>
+      </c>
+      <c r="H17" s="36" t="str">
         <f>IF($C17=ML,"X","")</f>
         <v/>
       </c>
-      <c r="I17" s="35" t="str">
+      <c r="I17" s="36" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="J17" s="35" t="str">
+      <c r="J17" s="36" t="str">
         <f>IF($C17=NL,"X","")</f>
         <v/>
       </c>
-      <c r="K17" s="35" t="str">
+      <c r="K17" s="36" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
     </row>
     <row r="18" outlineLevel="1">
-      <c r="A18" s="28"/>
-      <c r="B18" s="31" t="str">
+      <c r="A18" s="31"/>
+      <c r="B18" s="34" t="str">
         <f>RUBRICA!A9</f>
         <v>6. Entrega la documentación y evidencias requerida por la asignatura de acuerdo a la estrucutra y nombres solicitados, guardando todas las evidencias de avances en Git</v>
       </c>
-      <c r="C18" s="33" t="s">
-        <v>24</v>
-      </c>
-      <c r="D18" s="35" t="str">
+      <c r="C18" s="35" t="s">
+        <v>60</v>
+      </c>
+      <c r="D18" s="36" t="str">
         <f>IF($C18=CL,"X","")</f>
+        <v/>
+      </c>
+      <c r="E18" s="36" t="str">
+        <f>IF(D18="X",100*0.2,"")</f>
+        <v/>
+      </c>
+      <c r="F18" s="36" t="str">
+        <f>IF($C18=L,"X","")</f>
         <v>X</v>
       </c>
-      <c r="E18" s="35">
-        <f>IF(D18="X",100*0.2,"")</f>
-        <v>20</v>
-      </c>
-      <c r="F18" s="35" t="str">
-        <f>IF($C18=L,"X","")</f>
-        <v/>
-      </c>
-      <c r="G18" s="35" t="str">
+      <c r="G18" s="36">
         <f>IF(F18="X",60*0.2,"")</f>
-        <v/>
-      </c>
-      <c r="H18" s="35" t="str">
+        <v>12</v>
+      </c>
+      <c r="H18" s="36" t="str">
         <f>IF($C18=ML,"X","")</f>
         <v/>
       </c>
-      <c r="I18" s="35" t="str">
+      <c r="I18" s="36" t="str">
         <f>IF(H18="X",30*0.2,"")</f>
         <v/>
       </c>
-      <c r="J18" s="35" t="str">
+      <c r="J18" s="36" t="str">
         <f>IF($C18=NL,"X","")</f>
         <v/>
       </c>
-      <c r="K18" s="35" t="str">
+      <c r="K18" s="36" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
     </row>
     <row r="19" outlineLevel="1">
-      <c r="A19" s="28"/>
-      <c r="B19" s="31" t="str">
+      <c r="A19" s="31"/>
+      <c r="B19" s="34" t="str">
         <f>RUBRICA!A10</f>
         <v>7.- Generan evidencias claras dentro del repositorio  del aporte de cada uno de los integrantes del equipo que permitan identificar la equidad en el trabajo y la participación de cada estudiante.</v>
       </c>
-      <c r="C19" s="33" t="s">
-        <v>24</v>
-      </c>
-      <c r="D19" s="35" t="str">
+      <c r="C19" s="35" t="s">
+        <v>60</v>
+      </c>
+      <c r="D19" s="36" t="str">
         <f>IF($C19=CL,"X","")</f>
+        <v/>
+      </c>
+      <c r="E19" s="36" t="str">
+        <f>IF(D19="X",100*0.15,"")</f>
+        <v/>
+      </c>
+      <c r="F19" s="36" t="str">
+        <f>IF($C19=L,"X","")</f>
         <v>X</v>
       </c>
-      <c r="E19" s="35">
-        <f>IF(D19="X",100*0.15,"")</f>
-        <v>15</v>
-      </c>
-      <c r="F19" s="35" t="str">
-        <f>IF($C19=L,"X","")</f>
-        <v/>
-      </c>
-      <c r="G19" s="35" t="str">
+      <c r="G19" s="36">
         <f>IF(F19="X",60*0.15,"")</f>
-        <v/>
-      </c>
-      <c r="H19" s="35" t="str">
+        <v>9</v>
+      </c>
+      <c r="H19" s="36" t="str">
         <f>IF($C19=ML,"X","")</f>
         <v/>
       </c>
-      <c r="I19" s="35" t="str">
+      <c r="I19" s="36" t="str">
         <f>IF(H19="X",30*0.15,"")</f>
         <v/>
       </c>
-      <c r="J19" s="35" t="str">
+      <c r="J19" s="36" t="str">
         <f>IF($C19=NL,"X","")</f>
         <v/>
       </c>
-      <c r="K19" s="35" t="str">
+      <c r="K19" s="36" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
     </row>
     <row r="20" outlineLevel="1">
-      <c r="A20" s="28"/>
-      <c r="B20" s="31" t="str">
+      <c r="A20" s="31"/>
+      <c r="B20" s="34" t="str">
         <f>RUBRICA!A11</f>
         <v>8. Demuestra un trabajo en equipo en donde todos los miembros del equipo expresan con fluidez el conocimiento del tema expuesto y  participan de las actividades planificadas en el proyecto</v>
       </c>
-      <c r="C20" s="33" t="s">
-        <v>24</v>
-      </c>
-      <c r="D20" s="35" t="str">
+      <c r="C20" s="37" t="s">
+        <v>59</v>
+      </c>
+      <c r="D20" s="36" t="str">
         <f>IF($C20=CL,"X","")</f>
         <v>X</v>
       </c>
-      <c r="E20" s="35">
+      <c r="E20" s="36">
         <f>IF(D20="X",100*0.1,"")</f>
         <v>10</v>
       </c>
-      <c r="F20" s="35" t="str">
+      <c r="F20" s="36" t="str">
         <f>IF($C20=L,"X","")</f>
         <v/>
       </c>
-      <c r="G20" s="35" t="str">
+      <c r="G20" s="36" t="str">
         <f>IF(F20="X",60*0.1,"")</f>
         <v/>
       </c>
-      <c r="H20" s="35" t="str">
+      <c r="H20" s="36" t="str">
         <f>IF($C20=ML,"X","")</f>
         <v/>
       </c>
-      <c r="I20" s="35" t="str">
+      <c r="I20" s="36" t="str">
         <f>IF(H20="X",30*0.1,"")</f>
         <v/>
       </c>
-      <c r="J20" s="35" t="str">
+      <c r="J20" s="36" t="str">
         <f>IF($C20=NL,"X","")</f>
         <v/>
       </c>
-      <c r="K20" s="35" t="str">
+      <c r="K20" s="36" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1" outlineLevel="1">
-      <c r="A21" s="28"/>
+      <c r="A21" s="31"/>
       <c r="B21" s="48" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C21" s="49">
         <f>E21+G21+I21+K21</f>
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="D21" s="50"/>
       <c r="E21" s="50">
         <f>SUM(E13:E20)</f>
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="F21" s="50"/>
       <c r="G21" s="50">
         <f>SUM(G13:G20)</f>
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="H21" s="50"/>
       <c r="I21" s="50">
@@ -1511,18 +1523,18 @@
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1" outlineLevel="1">
-      <c r="A22" s="30"/>
+      <c r="A22" s="33"/>
       <c r="B22" s="51" t="s">
         <v>3</v>
       </c>
       <c r="C22" s="52">
         <f>VLOOKUP(C21,ESCALA_IEP!A2:B202,2,FALSE)</f>
-        <v>7</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="D23" s="1" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="24" ht="48.0" customHeight="1">
@@ -2553,208 +2565,207 @@
   <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0" outlineLevelRow="1"/>
   <cols>
     <col customWidth="1" min="1" max="6" width="38.71"/>
-    <col customWidth="1" min="7" max="26" width="11.43"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
-      <c r="A1" s="5" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="5" t="s">
+      <c r="A1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="3" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="12"/>
       <c r="B2" s="13" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C2" s="13" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D2" s="15" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E2" s="16" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F2" s="12"/>
     </row>
     <row r="3" ht="14.25" customHeight="1">
-      <c r="A3" s="17"/>
-      <c r="B3" s="17"/>
-      <c r="C3" s="17"/>
-      <c r="D3" s="18">
+      <c r="A3" s="12"/>
+      <c r="B3" s="12"/>
+      <c r="C3" s="12"/>
+      <c r="D3" s="17">
         <v>-0.3</v>
       </c>
-      <c r="E3" s="18">
+      <c r="E3" s="17">
         <v>0.0</v>
       </c>
-      <c r="F3" s="19"/>
+      <c r="F3" s="18"/>
     </row>
     <row r="4" ht="14.25" customHeight="1">
-      <c r="A4" s="21" t="s">
-        <v>13</v>
-      </c>
-      <c r="B4" s="21" t="s">
-        <v>14</v>
-      </c>
-      <c r="C4" s="21" t="s">
-        <v>16</v>
-      </c>
-      <c r="D4" s="21" t="s">
+      <c r="A4" s="19" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="E4" s="21" t="s">
+      <c r="C4" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="F4" s="25">
+      <c r="E4" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="F4" s="20">
         <v>10.0</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
-      <c r="A5" s="21" t="s">
-        <v>20</v>
-      </c>
-      <c r="B5" s="21" t="s">
+      <c r="A5" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="C5" s="21" t="s">
+      <c r="B5" s="19" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="D5" s="21" t="s">
+      <c r="D5" s="19" t="s">
+        <v>24</v>
+      </c>
+      <c r="E5" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="E5" s="21" t="s">
+      <c r="F5" s="20">
+        <v>10.0</v>
+      </c>
+    </row>
+    <row r="6" ht="14.25" customHeight="1">
+      <c r="A6" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="F5" s="25">
-        <v>10.0</v>
-      </c>
-    </row>
-    <row r="6" ht="14.25" customHeight="1">
-      <c r="A6" s="21" t="s">
+      <c r="B6" s="19" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="19" t="s">
         <v>28</v>
       </c>
-      <c r="B6" s="21" t="s">
+      <c r="D6" s="19" t="s">
+        <v>29</v>
+      </c>
+      <c r="E6" s="19" t="s">
         <v>30</v>
       </c>
-      <c r="C6" s="21" t="s">
+      <c r="F6" s="20">
+        <v>25.0</v>
+      </c>
+    </row>
+    <row r="7" ht="14.25" customHeight="1">
+      <c r="A7" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="D6" s="21" t="s">
+      <c r="B7" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="E6" s="21" t="s">
+      <c r="C7" s="19" t="s">
         <v>33</v>
       </c>
-      <c r="F6" s="25">
-        <v>25.0</v>
-      </c>
-    </row>
-    <row r="7" ht="14.25" customHeight="1">
-      <c r="A7" s="21" t="s">
+      <c r="D7" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="B7" s="21" t="s">
+      <c r="E7" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="C7" s="21" t="s">
+      <c r="F7" s="20">
+        <v>5.0</v>
+      </c>
+    </row>
+    <row r="8" ht="14.25" customHeight="1">
+      <c r="A8" s="19" t="s">
         <v>36</v>
       </c>
-      <c r="D7" s="21" t="s">
+      <c r="B8" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="E7" s="21" t="s">
+      <c r="C8" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="F7" s="25">
+      <c r="D8" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="E8" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="F8" s="21">
         <v>5.0</v>
       </c>
     </row>
-    <row r="8" ht="14.25" customHeight="1">
-      <c r="A8" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="B8" s="21" t="s">
-        <v>40</v>
-      </c>
-      <c r="C8" s="21" t="s">
+    <row r="9" ht="14.25" customHeight="1">
+      <c r="A9" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="D8" s="21" t="s">
+      <c r="B9" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="E8" s="21" t="s">
+      <c r="C9" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="F8" s="32">
-        <v>5.0</v>
-      </c>
-    </row>
-    <row r="9" ht="14.25" customHeight="1">
-      <c r="A9" s="21" t="s">
+      <c r="D9" s="19" t="s">
         <v>44</v>
       </c>
-      <c r="B9" s="21" t="s">
+      <c r="E9" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="C9" s="21" t="s">
+      <c r="F9" s="20">
+        <v>20.0</v>
+      </c>
+    </row>
+    <row r="10" ht="14.25" customHeight="1">
+      <c r="A10" s="23" t="s">
         <v>46</v>
       </c>
-      <c r="D9" s="21" t="s">
+      <c r="B10" s="23" t="s">
         <v>47</v>
       </c>
-      <c r="E9" s="21" t="s">
+      <c r="C10" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="F9" s="25">
-        <v>20.0</v>
-      </c>
-    </row>
-    <row r="10" ht="14.25" customHeight="1">
-      <c r="A10" s="34" t="s">
+      <c r="D10" s="23" t="s">
         <v>49</v>
       </c>
-      <c r="B10" s="34" t="s">
+      <c r="E10" s="23" t="s">
         <v>50</v>
       </c>
-      <c r="C10" s="34" t="s">
-        <v>51</v>
-      </c>
-      <c r="D10" s="34" t="s">
+      <c r="F10" s="25">
+        <v>15.0</v>
+      </c>
+    </row>
+    <row r="11" ht="81.0" customHeight="1">
+      <c r="A11" s="19" t="s">
         <v>52</v>
       </c>
-      <c r="E10" s="34" t="s">
+      <c r="B11" s="19" t="s">
         <v>53</v>
       </c>
-      <c r="F10" s="36">
-        <v>15.0</v>
-      </c>
-    </row>
-    <row r="11" ht="81.0" customHeight="1">
-      <c r="A11" s="21" t="s">
+      <c r="C11" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="B11" s="21" t="s">
+      <c r="D11" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="C11" s="21" t="s">
-        <v>56</v>
-      </c>
-      <c r="D11" s="21" t="s">
+      <c r="E11" s="19" t="s">
         <v>57</v>
       </c>
-      <c r="E11" s="21" t="s">
-        <v>58</v>
-      </c>
-      <c r="F11" s="37">
+      <c r="F11" s="27">
         <v>10.0</v>
       </c>
     </row>
@@ -2967,786 +2978,786 @@
     <row r="218" ht="14.25" customHeight="1"/>
     <row r="219" ht="14.25" customHeight="1"/>
     <row r="220" ht="14.25" customHeight="1"/>
-    <row r="221" ht="14.25" customHeight="1"/>
-    <row r="222" ht="14.25" customHeight="1"/>
-    <row r="223" ht="14.25" customHeight="1"/>
-    <row r="224" ht="14.25" customHeight="1"/>
-    <row r="225" ht="14.25" customHeight="1"/>
-    <row r="226" ht="14.25" customHeight="1"/>
-    <row r="227" ht="14.25" customHeight="1"/>
-    <row r="228" ht="14.25" customHeight="1"/>
-    <row r="229" ht="14.25" customHeight="1"/>
-    <row r="230" ht="14.25" customHeight="1"/>
-    <row r="231" ht="14.25" customHeight="1"/>
-    <row r="232" ht="14.25" customHeight="1"/>
-    <row r="233" ht="14.25" customHeight="1"/>
-    <row r="234" ht="14.25" customHeight="1"/>
-    <row r="235" ht="14.25" customHeight="1"/>
-    <row r="236" ht="14.25" customHeight="1"/>
-    <row r="237" ht="14.25" customHeight="1"/>
-    <row r="238" ht="14.25" customHeight="1"/>
-    <row r="239" ht="14.25" customHeight="1"/>
-    <row r="240" ht="14.25" customHeight="1"/>
-    <row r="241" ht="14.25" customHeight="1"/>
-    <row r="242" ht="14.25" customHeight="1"/>
-    <row r="243" ht="14.25" customHeight="1"/>
-    <row r="244" ht="14.25" customHeight="1"/>
-    <row r="245" ht="14.25" customHeight="1"/>
-    <row r="246" ht="14.25" customHeight="1"/>
-    <row r="247" ht="14.25" customHeight="1"/>
-    <row r="248" ht="14.25" customHeight="1"/>
-    <row r="249" ht="14.25" customHeight="1"/>
-    <row r="250" ht="14.25" customHeight="1"/>
-    <row r="251" ht="14.25" customHeight="1"/>
-    <row r="252" ht="14.25" customHeight="1"/>
-    <row r="253" ht="14.25" customHeight="1"/>
-    <row r="254" ht="14.25" customHeight="1"/>
-    <row r="255" ht="14.25" customHeight="1"/>
-    <row r="256" ht="14.25" customHeight="1"/>
-    <row r="257" ht="14.25" customHeight="1"/>
-    <row r="258" ht="14.25" customHeight="1"/>
-    <row r="259" ht="14.25" customHeight="1"/>
-    <row r="260" ht="14.25" customHeight="1"/>
-    <row r="261" ht="14.25" customHeight="1"/>
-    <row r="262" ht="14.25" customHeight="1"/>
-    <row r="263" ht="14.25" customHeight="1"/>
-    <row r="264" ht="14.25" customHeight="1"/>
-    <row r="265" ht="14.25" customHeight="1"/>
-    <row r="266" ht="14.25" customHeight="1"/>
-    <row r="267" ht="14.25" customHeight="1"/>
-    <row r="268" ht="14.25" customHeight="1"/>
-    <row r="269" ht="14.25" customHeight="1"/>
-    <row r="270" ht="14.25" customHeight="1"/>
-    <row r="271" ht="14.25" customHeight="1"/>
-    <row r="272" ht="14.25" customHeight="1"/>
-    <row r="273" ht="14.25" customHeight="1"/>
-    <row r="274" ht="14.25" customHeight="1"/>
-    <row r="275" ht="14.25" customHeight="1"/>
-    <row r="276" ht="14.25" customHeight="1"/>
-    <row r="277" ht="14.25" customHeight="1"/>
-    <row r="278" ht="14.25" customHeight="1"/>
-    <row r="279" ht="14.25" customHeight="1"/>
-    <row r="280" ht="14.25" customHeight="1"/>
-    <row r="281" ht="14.25" customHeight="1"/>
-    <row r="282" ht="14.25" customHeight="1"/>
-    <row r="283" ht="14.25" customHeight="1"/>
-    <row r="284" ht="14.25" customHeight="1"/>
-    <row r="285" ht="14.25" customHeight="1"/>
-    <row r="286" ht="14.25" customHeight="1"/>
-    <row r="287" ht="14.25" customHeight="1"/>
-    <row r="288" ht="14.25" customHeight="1"/>
-    <row r="289" ht="14.25" customHeight="1"/>
-    <row r="290" ht="14.25" customHeight="1"/>
-    <row r="291" ht="14.25" customHeight="1"/>
-    <row r="292" ht="14.25" customHeight="1"/>
-    <row r="293" ht="14.25" customHeight="1"/>
-    <row r="294" ht="14.25" customHeight="1"/>
-    <row r="295" ht="14.25" customHeight="1"/>
-    <row r="296" ht="14.25" customHeight="1"/>
-    <row r="297" ht="14.25" customHeight="1"/>
-    <row r="298" ht="14.25" customHeight="1"/>
-    <row r="299" ht="14.25" customHeight="1"/>
-    <row r="300" ht="14.25" customHeight="1"/>
-    <row r="301" ht="14.25" customHeight="1"/>
-    <row r="302" ht="14.25" customHeight="1"/>
-    <row r="303" ht="14.25" customHeight="1"/>
-    <row r="304" ht="14.25" customHeight="1"/>
-    <row r="305" ht="14.25" customHeight="1"/>
-    <row r="306" ht="14.25" customHeight="1"/>
-    <row r="307" ht="14.25" customHeight="1"/>
-    <row r="308" ht="14.25" customHeight="1"/>
-    <row r="309" ht="14.25" customHeight="1"/>
-    <row r="310" ht="14.25" customHeight="1"/>
-    <row r="311" ht="14.25" customHeight="1"/>
-    <row r="312" ht="14.25" customHeight="1"/>
-    <row r="313" ht="14.25" customHeight="1"/>
-    <row r="314" ht="14.25" customHeight="1"/>
-    <row r="315" ht="14.25" customHeight="1"/>
-    <row r="316" ht="14.25" customHeight="1"/>
-    <row r="317" ht="14.25" customHeight="1"/>
-    <row r="318" ht="14.25" customHeight="1"/>
-    <row r="319" ht="14.25" customHeight="1"/>
-    <row r="320" ht="14.25" customHeight="1"/>
-    <row r="321" ht="14.25" customHeight="1"/>
-    <row r="322" ht="14.25" customHeight="1"/>
-    <row r="323" ht="14.25" customHeight="1"/>
-    <row r="324" ht="14.25" customHeight="1"/>
-    <row r="325" ht="14.25" customHeight="1"/>
-    <row r="326" ht="14.25" customHeight="1"/>
-    <row r="327" ht="14.25" customHeight="1"/>
-    <row r="328" ht="14.25" customHeight="1"/>
-    <row r="329" ht="14.25" customHeight="1"/>
-    <row r="330" ht="14.25" customHeight="1"/>
-    <row r="331" ht="14.25" customHeight="1"/>
-    <row r="332" ht="14.25" customHeight="1"/>
-    <row r="333" ht="14.25" customHeight="1"/>
-    <row r="334" ht="14.25" customHeight="1"/>
-    <row r="335" ht="14.25" customHeight="1"/>
-    <row r="336" ht="14.25" customHeight="1"/>
-    <row r="337" ht="14.25" customHeight="1"/>
-    <row r="338" ht="14.25" customHeight="1"/>
-    <row r="339" ht="14.25" customHeight="1"/>
-    <row r="340" ht="14.25" customHeight="1"/>
-    <row r="341" ht="14.25" customHeight="1"/>
-    <row r="342" ht="14.25" customHeight="1"/>
-    <row r="343" ht="14.25" customHeight="1"/>
-    <row r="344" ht="14.25" customHeight="1"/>
-    <row r="345" ht="14.25" customHeight="1"/>
-    <row r="346" ht="14.25" customHeight="1"/>
-    <row r="347" ht="14.25" customHeight="1"/>
-    <row r="348" ht="14.25" customHeight="1"/>
-    <row r="349" ht="14.25" customHeight="1"/>
-    <row r="350" ht="14.25" customHeight="1"/>
-    <row r="351" ht="14.25" customHeight="1"/>
-    <row r="352" ht="14.25" customHeight="1"/>
-    <row r="353" ht="14.25" customHeight="1"/>
-    <row r="354" ht="14.25" customHeight="1"/>
-    <row r="355" ht="14.25" customHeight="1"/>
-    <row r="356" ht="14.25" customHeight="1"/>
-    <row r="357" ht="14.25" customHeight="1"/>
-    <row r="358" ht="14.25" customHeight="1"/>
-    <row r="359" ht="14.25" customHeight="1"/>
-    <row r="360" ht="14.25" customHeight="1"/>
-    <row r="361" ht="14.25" customHeight="1"/>
-    <row r="362" ht="14.25" customHeight="1"/>
-    <row r="363" ht="14.25" customHeight="1"/>
-    <row r="364" ht="14.25" customHeight="1"/>
-    <row r="365" ht="14.25" customHeight="1"/>
-    <row r="366" ht="14.25" customHeight="1"/>
-    <row r="367" ht="14.25" customHeight="1"/>
-    <row r="368" ht="14.25" customHeight="1"/>
-    <row r="369" ht="14.25" customHeight="1"/>
-    <row r="370" ht="14.25" customHeight="1"/>
-    <row r="371" ht="14.25" customHeight="1"/>
-    <row r="372" ht="14.25" customHeight="1"/>
-    <row r="373" ht="14.25" customHeight="1"/>
-    <row r="374" ht="14.25" customHeight="1"/>
-    <row r="375" ht="14.25" customHeight="1"/>
-    <row r="376" ht="14.25" customHeight="1"/>
-    <row r="377" ht="14.25" customHeight="1"/>
-    <row r="378" ht="14.25" customHeight="1"/>
-    <row r="379" ht="14.25" customHeight="1"/>
-    <row r="380" ht="14.25" customHeight="1"/>
-    <row r="381" ht="14.25" customHeight="1"/>
-    <row r="382" ht="14.25" customHeight="1"/>
-    <row r="383" ht="14.25" customHeight="1"/>
-    <row r="384" ht="14.25" customHeight="1"/>
-    <row r="385" ht="14.25" customHeight="1"/>
-    <row r="386" ht="14.25" customHeight="1"/>
-    <row r="387" ht="14.25" customHeight="1"/>
-    <row r="388" ht="14.25" customHeight="1"/>
-    <row r="389" ht="14.25" customHeight="1"/>
-    <row r="390" ht="14.25" customHeight="1"/>
-    <row r="391" ht="14.25" customHeight="1"/>
-    <row r="392" ht="14.25" customHeight="1"/>
-    <row r="393" ht="14.25" customHeight="1"/>
-    <row r="394" ht="14.25" customHeight="1"/>
-    <row r="395" ht="14.25" customHeight="1"/>
-    <row r="396" ht="14.25" customHeight="1"/>
-    <row r="397" ht="14.25" customHeight="1"/>
-    <row r="398" ht="14.25" customHeight="1"/>
-    <row r="399" ht="14.25" customHeight="1"/>
-    <row r="400" ht="14.25" customHeight="1"/>
-    <row r="401" ht="14.25" customHeight="1"/>
-    <row r="402" ht="14.25" customHeight="1"/>
-    <row r="403" ht="14.25" customHeight="1"/>
-    <row r="404" ht="14.25" customHeight="1"/>
-    <row r="405" ht="14.25" customHeight="1"/>
-    <row r="406" ht="14.25" customHeight="1"/>
-    <row r="407" ht="14.25" customHeight="1"/>
-    <row r="408" ht="14.25" customHeight="1"/>
-    <row r="409" ht="14.25" customHeight="1"/>
-    <row r="410" ht="14.25" customHeight="1"/>
-    <row r="411" ht="14.25" customHeight="1"/>
-    <row r="412" ht="14.25" customHeight="1"/>
-    <row r="413" ht="14.25" customHeight="1"/>
-    <row r="414" ht="14.25" customHeight="1"/>
-    <row r="415" ht="14.25" customHeight="1"/>
-    <row r="416" ht="14.25" customHeight="1"/>
-    <row r="417" ht="14.25" customHeight="1"/>
-    <row r="418" ht="14.25" customHeight="1"/>
-    <row r="419" ht="14.25" customHeight="1"/>
-    <row r="420" ht="14.25" customHeight="1"/>
-    <row r="421" ht="14.25" customHeight="1"/>
-    <row r="422" ht="14.25" customHeight="1"/>
-    <row r="423" ht="14.25" customHeight="1"/>
-    <row r="424" ht="14.25" customHeight="1"/>
-    <row r="425" ht="14.25" customHeight="1"/>
-    <row r="426" ht="14.25" customHeight="1"/>
-    <row r="427" ht="14.25" customHeight="1"/>
-    <row r="428" ht="14.25" customHeight="1"/>
-    <row r="429" ht="14.25" customHeight="1"/>
-    <row r="430" ht="14.25" customHeight="1"/>
-    <row r="431" ht="14.25" customHeight="1"/>
-    <row r="432" ht="14.25" customHeight="1"/>
-    <row r="433" ht="14.25" customHeight="1"/>
-    <row r="434" ht="14.25" customHeight="1"/>
-    <row r="435" ht="14.25" customHeight="1"/>
-    <row r="436" ht="14.25" customHeight="1"/>
-    <row r="437" ht="14.25" customHeight="1"/>
-    <row r="438" ht="14.25" customHeight="1"/>
-    <row r="439" ht="14.25" customHeight="1"/>
-    <row r="440" ht="14.25" customHeight="1"/>
-    <row r="441" ht="14.25" customHeight="1"/>
-    <row r="442" ht="14.25" customHeight="1"/>
-    <row r="443" ht="14.25" customHeight="1"/>
-    <row r="444" ht="14.25" customHeight="1"/>
-    <row r="445" ht="14.25" customHeight="1"/>
-    <row r="446" ht="14.25" customHeight="1"/>
-    <row r="447" ht="14.25" customHeight="1"/>
-    <row r="448" ht="14.25" customHeight="1"/>
-    <row r="449" ht="14.25" customHeight="1"/>
-    <row r="450" ht="14.25" customHeight="1"/>
-    <row r="451" ht="14.25" customHeight="1"/>
-    <row r="452" ht="14.25" customHeight="1"/>
-    <row r="453" ht="14.25" customHeight="1"/>
-    <row r="454" ht="14.25" customHeight="1"/>
-    <row r="455" ht="14.25" customHeight="1"/>
-    <row r="456" ht="14.25" customHeight="1"/>
-    <row r="457" ht="14.25" customHeight="1"/>
-    <row r="458" ht="14.25" customHeight="1"/>
-    <row r="459" ht="14.25" customHeight="1"/>
-    <row r="460" ht="14.25" customHeight="1"/>
-    <row r="461" ht="14.25" customHeight="1"/>
-    <row r="462" ht="14.25" customHeight="1"/>
-    <row r="463" ht="14.25" customHeight="1"/>
-    <row r="464" ht="14.25" customHeight="1"/>
-    <row r="465" ht="14.25" customHeight="1"/>
-    <row r="466" ht="14.25" customHeight="1"/>
-    <row r="467" ht="14.25" customHeight="1"/>
-    <row r="468" ht="14.25" customHeight="1"/>
-    <row r="469" ht="14.25" customHeight="1"/>
-    <row r="470" ht="14.25" customHeight="1"/>
-    <row r="471" ht="14.25" customHeight="1"/>
-    <row r="472" ht="14.25" customHeight="1"/>
-    <row r="473" ht="14.25" customHeight="1"/>
-    <row r="474" ht="14.25" customHeight="1"/>
-    <row r="475" ht="14.25" customHeight="1"/>
-    <row r="476" ht="14.25" customHeight="1"/>
-    <row r="477" ht="14.25" customHeight="1"/>
-    <row r="478" ht="14.25" customHeight="1"/>
-    <row r="479" ht="14.25" customHeight="1"/>
-    <row r="480" ht="14.25" customHeight="1"/>
-    <row r="481" ht="14.25" customHeight="1"/>
-    <row r="482" ht="14.25" customHeight="1"/>
-    <row r="483" ht="14.25" customHeight="1"/>
-    <row r="484" ht="14.25" customHeight="1"/>
-    <row r="485" ht="14.25" customHeight="1"/>
-    <row r="486" ht="14.25" customHeight="1"/>
-    <row r="487" ht="14.25" customHeight="1"/>
-    <row r="488" ht="14.25" customHeight="1"/>
-    <row r="489" ht="14.25" customHeight="1"/>
-    <row r="490" ht="14.25" customHeight="1"/>
-    <row r="491" ht="14.25" customHeight="1"/>
-    <row r="492" ht="14.25" customHeight="1"/>
-    <row r="493" ht="14.25" customHeight="1"/>
-    <row r="494" ht="14.25" customHeight="1"/>
-    <row r="495" ht="14.25" customHeight="1"/>
-    <row r="496" ht="14.25" customHeight="1"/>
-    <row r="497" ht="14.25" customHeight="1"/>
-    <row r="498" ht="14.25" customHeight="1"/>
-    <row r="499" ht="14.25" customHeight="1"/>
-    <row r="500" ht="14.25" customHeight="1"/>
-    <row r="501" ht="14.25" customHeight="1"/>
-    <row r="502" ht="14.25" customHeight="1"/>
-    <row r="503" ht="14.25" customHeight="1"/>
-    <row r="504" ht="14.25" customHeight="1"/>
-    <row r="505" ht="14.25" customHeight="1"/>
-    <row r="506" ht="14.25" customHeight="1"/>
-    <row r="507" ht="14.25" customHeight="1"/>
-    <row r="508" ht="14.25" customHeight="1"/>
-    <row r="509" ht="14.25" customHeight="1"/>
-    <row r="510" ht="14.25" customHeight="1"/>
-    <row r="511" ht="14.25" customHeight="1"/>
-    <row r="512" ht="14.25" customHeight="1"/>
-    <row r="513" ht="14.25" customHeight="1"/>
-    <row r="514" ht="14.25" customHeight="1"/>
-    <row r="515" ht="14.25" customHeight="1"/>
-    <row r="516" ht="14.25" customHeight="1"/>
-    <row r="517" ht="14.25" customHeight="1"/>
-    <row r="518" ht="14.25" customHeight="1"/>
-    <row r="519" ht="14.25" customHeight="1"/>
-    <row r="520" ht="14.25" customHeight="1"/>
-    <row r="521" ht="14.25" customHeight="1"/>
-    <row r="522" ht="14.25" customHeight="1"/>
-    <row r="523" ht="14.25" customHeight="1"/>
-    <row r="524" ht="14.25" customHeight="1"/>
-    <row r="525" ht="14.25" customHeight="1"/>
-    <row r="526" ht="14.25" customHeight="1"/>
-    <row r="527" ht="14.25" customHeight="1"/>
-    <row r="528" ht="14.25" customHeight="1"/>
-    <row r="529" ht="14.25" customHeight="1"/>
-    <row r="530" ht="14.25" customHeight="1"/>
-    <row r="531" ht="14.25" customHeight="1"/>
-    <row r="532" ht="14.25" customHeight="1"/>
-    <row r="533" ht="14.25" customHeight="1"/>
-    <row r="534" ht="14.25" customHeight="1"/>
-    <row r="535" ht="14.25" customHeight="1"/>
-    <row r="536" ht="14.25" customHeight="1"/>
-    <row r="537" ht="14.25" customHeight="1"/>
-    <row r="538" ht="14.25" customHeight="1"/>
-    <row r="539" ht="14.25" customHeight="1"/>
-    <row r="540" ht="14.25" customHeight="1"/>
-    <row r="541" ht="14.25" customHeight="1"/>
-    <row r="542" ht="14.25" customHeight="1"/>
-    <row r="543" ht="14.25" customHeight="1"/>
-    <row r="544" ht="14.25" customHeight="1"/>
-    <row r="545" ht="14.25" customHeight="1"/>
-    <row r="546" ht="14.25" customHeight="1"/>
-    <row r="547" ht="14.25" customHeight="1"/>
-    <row r="548" ht="14.25" customHeight="1"/>
-    <row r="549" ht="14.25" customHeight="1"/>
-    <row r="550" ht="14.25" customHeight="1"/>
-    <row r="551" ht="14.25" customHeight="1"/>
-    <row r="552" ht="14.25" customHeight="1"/>
-    <row r="553" ht="14.25" customHeight="1"/>
-    <row r="554" ht="14.25" customHeight="1"/>
-    <row r="555" ht="14.25" customHeight="1"/>
-    <row r="556" ht="14.25" customHeight="1"/>
-    <row r="557" ht="14.25" customHeight="1"/>
-    <row r="558" ht="14.25" customHeight="1"/>
-    <row r="559" ht="14.25" customHeight="1"/>
-    <row r="560" ht="14.25" customHeight="1"/>
-    <row r="561" ht="14.25" customHeight="1"/>
-    <row r="562" ht="14.25" customHeight="1"/>
-    <row r="563" ht="14.25" customHeight="1"/>
-    <row r="564" ht="14.25" customHeight="1"/>
-    <row r="565" ht="14.25" customHeight="1"/>
-    <row r="566" ht="14.25" customHeight="1"/>
-    <row r="567" ht="14.25" customHeight="1"/>
-    <row r="568" ht="14.25" customHeight="1"/>
-    <row r="569" ht="14.25" customHeight="1"/>
-    <row r="570" ht="14.25" customHeight="1"/>
-    <row r="571" ht="14.25" customHeight="1"/>
-    <row r="572" ht="14.25" customHeight="1"/>
-    <row r="573" ht="14.25" customHeight="1"/>
-    <row r="574" ht="14.25" customHeight="1"/>
-    <row r="575" ht="14.25" customHeight="1"/>
-    <row r="576" ht="14.25" customHeight="1"/>
-    <row r="577" ht="14.25" customHeight="1"/>
-    <row r="578" ht="14.25" customHeight="1"/>
-    <row r="579" ht="14.25" customHeight="1"/>
-    <row r="580" ht="14.25" customHeight="1"/>
-    <row r="581" ht="14.25" customHeight="1"/>
-    <row r="582" ht="14.25" customHeight="1"/>
-    <row r="583" ht="14.25" customHeight="1"/>
-    <row r="584" ht="14.25" customHeight="1"/>
-    <row r="585" ht="14.25" customHeight="1"/>
-    <row r="586" ht="14.25" customHeight="1"/>
-    <row r="587" ht="14.25" customHeight="1"/>
-    <row r="588" ht="14.25" customHeight="1"/>
-    <row r="589" ht="14.25" customHeight="1"/>
-    <row r="590" ht="14.25" customHeight="1"/>
-    <row r="591" ht="14.25" customHeight="1"/>
-    <row r="592" ht="14.25" customHeight="1"/>
-    <row r="593" ht="14.25" customHeight="1"/>
-    <row r="594" ht="14.25" customHeight="1"/>
-    <row r="595" ht="14.25" customHeight="1"/>
-    <row r="596" ht="14.25" customHeight="1"/>
-    <row r="597" ht="14.25" customHeight="1"/>
-    <row r="598" ht="14.25" customHeight="1"/>
-    <row r="599" ht="14.25" customHeight="1"/>
-    <row r="600" ht="14.25" customHeight="1"/>
-    <row r="601" ht="14.25" customHeight="1"/>
-    <row r="602" ht="14.25" customHeight="1"/>
-    <row r="603" ht="14.25" customHeight="1"/>
-    <row r="604" ht="14.25" customHeight="1"/>
-    <row r="605" ht="14.25" customHeight="1"/>
-    <row r="606" ht="14.25" customHeight="1"/>
-    <row r="607" ht="14.25" customHeight="1"/>
-    <row r="608" ht="14.25" customHeight="1"/>
-    <row r="609" ht="14.25" customHeight="1"/>
-    <row r="610" ht="14.25" customHeight="1"/>
-    <row r="611" ht="14.25" customHeight="1"/>
-    <row r="612" ht="14.25" customHeight="1"/>
-    <row r="613" ht="14.25" customHeight="1"/>
-    <row r="614" ht="14.25" customHeight="1"/>
-    <row r="615" ht="14.25" customHeight="1"/>
-    <row r="616" ht="14.25" customHeight="1"/>
-    <row r="617" ht="14.25" customHeight="1"/>
-    <row r="618" ht="14.25" customHeight="1"/>
-    <row r="619" ht="14.25" customHeight="1"/>
-    <row r="620" ht="14.25" customHeight="1"/>
-    <row r="621" ht="14.25" customHeight="1"/>
-    <row r="622" ht="14.25" customHeight="1"/>
-    <row r="623" ht="14.25" customHeight="1"/>
-    <row r="624" ht="14.25" customHeight="1"/>
-    <row r="625" ht="14.25" customHeight="1"/>
-    <row r="626" ht="14.25" customHeight="1"/>
-    <row r="627" ht="14.25" customHeight="1"/>
-    <row r="628" ht="14.25" customHeight="1"/>
-    <row r="629" ht="14.25" customHeight="1"/>
-    <row r="630" ht="14.25" customHeight="1"/>
-    <row r="631" ht="14.25" customHeight="1"/>
-    <row r="632" ht="14.25" customHeight="1"/>
-    <row r="633" ht="14.25" customHeight="1"/>
-    <row r="634" ht="14.25" customHeight="1"/>
-    <row r="635" ht="14.25" customHeight="1"/>
-    <row r="636" ht="14.25" customHeight="1"/>
-    <row r="637" ht="14.25" customHeight="1"/>
-    <row r="638" ht="14.25" customHeight="1"/>
-    <row r="639" ht="14.25" customHeight="1"/>
-    <row r="640" ht="14.25" customHeight="1"/>
-    <row r="641" ht="14.25" customHeight="1"/>
-    <row r="642" ht="14.25" customHeight="1"/>
-    <row r="643" ht="14.25" customHeight="1"/>
-    <row r="644" ht="14.25" customHeight="1"/>
-    <row r="645" ht="14.25" customHeight="1"/>
-    <row r="646" ht="14.25" customHeight="1"/>
-    <row r="647" ht="14.25" customHeight="1"/>
-    <row r="648" ht="14.25" customHeight="1"/>
-    <row r="649" ht="14.25" customHeight="1"/>
-    <row r="650" ht="14.25" customHeight="1"/>
-    <row r="651" ht="14.25" customHeight="1"/>
-    <row r="652" ht="14.25" customHeight="1"/>
-    <row r="653" ht="14.25" customHeight="1"/>
-    <row r="654" ht="14.25" customHeight="1"/>
-    <row r="655" ht="14.25" customHeight="1"/>
-    <row r="656" ht="14.25" customHeight="1"/>
-    <row r="657" ht="14.25" customHeight="1"/>
-    <row r="658" ht="14.25" customHeight="1"/>
-    <row r="659" ht="14.25" customHeight="1"/>
-    <row r="660" ht="14.25" customHeight="1"/>
-    <row r="661" ht="14.25" customHeight="1"/>
-    <row r="662" ht="14.25" customHeight="1"/>
-    <row r="663" ht="14.25" customHeight="1"/>
-    <row r="664" ht="14.25" customHeight="1"/>
-    <row r="665" ht="14.25" customHeight="1"/>
-    <row r="666" ht="14.25" customHeight="1"/>
-    <row r="667" ht="14.25" customHeight="1"/>
-    <row r="668" ht="14.25" customHeight="1"/>
-    <row r="669" ht="14.25" customHeight="1"/>
-    <row r="670" ht="14.25" customHeight="1"/>
-    <row r="671" ht="14.25" customHeight="1"/>
-    <row r="672" ht="14.25" customHeight="1"/>
-    <row r="673" ht="14.25" customHeight="1"/>
-    <row r="674" ht="14.25" customHeight="1"/>
-    <row r="675" ht="14.25" customHeight="1"/>
-    <row r="676" ht="14.25" customHeight="1"/>
-    <row r="677" ht="14.25" customHeight="1"/>
-    <row r="678" ht="14.25" customHeight="1"/>
-    <row r="679" ht="14.25" customHeight="1"/>
-    <row r="680" ht="14.25" customHeight="1"/>
-    <row r="681" ht="14.25" customHeight="1"/>
-    <row r="682" ht="14.25" customHeight="1"/>
-    <row r="683" ht="14.25" customHeight="1"/>
-    <row r="684" ht="14.25" customHeight="1"/>
-    <row r="685" ht="14.25" customHeight="1"/>
-    <row r="686" ht="14.25" customHeight="1"/>
-    <row r="687" ht="14.25" customHeight="1"/>
-    <row r="688" ht="14.25" customHeight="1"/>
-    <row r="689" ht="14.25" customHeight="1"/>
-    <row r="690" ht="14.25" customHeight="1"/>
-    <row r="691" ht="14.25" customHeight="1"/>
-    <row r="692" ht="14.25" customHeight="1"/>
-    <row r="693" ht="14.25" customHeight="1"/>
-    <row r="694" ht="14.25" customHeight="1"/>
-    <row r="695" ht="14.25" customHeight="1"/>
-    <row r="696" ht="14.25" customHeight="1"/>
-    <row r="697" ht="14.25" customHeight="1"/>
-    <row r="698" ht="14.25" customHeight="1"/>
-    <row r="699" ht="14.25" customHeight="1"/>
-    <row r="700" ht="14.25" customHeight="1"/>
-    <row r="701" ht="14.25" customHeight="1"/>
-    <row r="702" ht="14.25" customHeight="1"/>
-    <row r="703" ht="14.25" customHeight="1"/>
-    <row r="704" ht="14.25" customHeight="1"/>
-    <row r="705" ht="14.25" customHeight="1"/>
-    <row r="706" ht="14.25" customHeight="1"/>
-    <row r="707" ht="14.25" customHeight="1"/>
-    <row r="708" ht="14.25" customHeight="1"/>
-    <row r="709" ht="14.25" customHeight="1"/>
-    <row r="710" ht="14.25" customHeight="1"/>
-    <row r="711" ht="14.25" customHeight="1"/>
-    <row r="712" ht="14.25" customHeight="1"/>
-    <row r="713" ht="14.25" customHeight="1"/>
-    <row r="714" ht="14.25" customHeight="1"/>
-    <row r="715" ht="14.25" customHeight="1"/>
-    <row r="716" ht="14.25" customHeight="1"/>
-    <row r="717" ht="14.25" customHeight="1"/>
-    <row r="718" ht="14.25" customHeight="1"/>
-    <row r="719" ht="14.25" customHeight="1"/>
-    <row r="720" ht="14.25" customHeight="1"/>
-    <row r="721" ht="14.25" customHeight="1"/>
-    <row r="722" ht="14.25" customHeight="1"/>
-    <row r="723" ht="14.25" customHeight="1"/>
-    <row r="724" ht="14.25" customHeight="1"/>
-    <row r="725" ht="14.25" customHeight="1"/>
-    <row r="726" ht="14.25" customHeight="1"/>
-    <row r="727" ht="14.25" customHeight="1"/>
-    <row r="728" ht="14.25" customHeight="1"/>
-    <row r="729" ht="14.25" customHeight="1"/>
-    <row r="730" ht="14.25" customHeight="1"/>
-    <row r="731" ht="14.25" customHeight="1"/>
-    <row r="732" ht="14.25" customHeight="1"/>
-    <row r="733" ht="14.25" customHeight="1"/>
-    <row r="734" ht="14.25" customHeight="1"/>
-    <row r="735" ht="14.25" customHeight="1"/>
-    <row r="736" ht="14.25" customHeight="1"/>
-    <row r="737" ht="14.25" customHeight="1"/>
-    <row r="738" ht="14.25" customHeight="1"/>
-    <row r="739" ht="14.25" customHeight="1"/>
-    <row r="740" ht="14.25" customHeight="1"/>
-    <row r="741" ht="14.25" customHeight="1"/>
-    <row r="742" ht="14.25" customHeight="1"/>
-    <row r="743" ht="14.25" customHeight="1"/>
-    <row r="744" ht="14.25" customHeight="1"/>
-    <row r="745" ht="14.25" customHeight="1"/>
-    <row r="746" ht="14.25" customHeight="1"/>
-    <row r="747" ht="14.25" customHeight="1"/>
-    <row r="748" ht="14.25" customHeight="1"/>
-    <row r="749" ht="14.25" customHeight="1"/>
-    <row r="750" ht="14.25" customHeight="1"/>
-    <row r="751" ht="14.25" customHeight="1"/>
-    <row r="752" ht="14.25" customHeight="1"/>
-    <row r="753" ht="14.25" customHeight="1"/>
-    <row r="754" ht="14.25" customHeight="1"/>
-    <row r="755" ht="14.25" customHeight="1"/>
-    <row r="756" ht="14.25" customHeight="1"/>
-    <row r="757" ht="14.25" customHeight="1"/>
-    <row r="758" ht="14.25" customHeight="1"/>
-    <row r="759" ht="14.25" customHeight="1"/>
-    <row r="760" ht="14.25" customHeight="1"/>
-    <row r="761" ht="14.25" customHeight="1"/>
-    <row r="762" ht="14.25" customHeight="1"/>
-    <row r="763" ht="14.25" customHeight="1"/>
-    <row r="764" ht="14.25" customHeight="1"/>
-    <row r="765" ht="14.25" customHeight="1"/>
-    <row r="766" ht="14.25" customHeight="1"/>
-    <row r="767" ht="14.25" customHeight="1"/>
-    <row r="768" ht="14.25" customHeight="1"/>
-    <row r="769" ht="14.25" customHeight="1"/>
-    <row r="770" ht="14.25" customHeight="1"/>
-    <row r="771" ht="14.25" customHeight="1"/>
-    <row r="772" ht="14.25" customHeight="1"/>
-    <row r="773" ht="14.25" customHeight="1"/>
-    <row r="774" ht="14.25" customHeight="1"/>
-    <row r="775" ht="14.25" customHeight="1"/>
-    <row r="776" ht="14.25" customHeight="1"/>
-    <row r="777" ht="14.25" customHeight="1"/>
-    <row r="778" ht="14.25" customHeight="1"/>
-    <row r="779" ht="14.25" customHeight="1"/>
-    <row r="780" ht="14.25" customHeight="1"/>
-    <row r="781" ht="14.25" customHeight="1"/>
-    <row r="782" ht="14.25" customHeight="1"/>
-    <row r="783" ht="14.25" customHeight="1"/>
-    <row r="784" ht="14.25" customHeight="1"/>
-    <row r="785" ht="14.25" customHeight="1"/>
-    <row r="786" ht="14.25" customHeight="1"/>
-    <row r="787" ht="14.25" customHeight="1"/>
-    <row r="788" ht="14.25" customHeight="1"/>
-    <row r="789" ht="14.25" customHeight="1"/>
-    <row r="790" ht="14.25" customHeight="1"/>
-    <row r="791" ht="14.25" customHeight="1"/>
-    <row r="792" ht="14.25" customHeight="1"/>
-    <row r="793" ht="14.25" customHeight="1"/>
-    <row r="794" ht="14.25" customHeight="1"/>
-    <row r="795" ht="14.25" customHeight="1"/>
-    <row r="796" ht="14.25" customHeight="1"/>
-    <row r="797" ht="14.25" customHeight="1"/>
-    <row r="798" ht="14.25" customHeight="1"/>
-    <row r="799" ht="14.25" customHeight="1"/>
-    <row r="800" ht="14.25" customHeight="1"/>
-    <row r="801" ht="14.25" customHeight="1"/>
-    <row r="802" ht="14.25" customHeight="1"/>
-    <row r="803" ht="14.25" customHeight="1"/>
-    <row r="804" ht="14.25" customHeight="1"/>
-    <row r="805" ht="14.25" customHeight="1"/>
-    <row r="806" ht="14.25" customHeight="1"/>
-    <row r="807" ht="14.25" customHeight="1"/>
-    <row r="808" ht="14.25" customHeight="1"/>
-    <row r="809" ht="14.25" customHeight="1"/>
-    <row r="810" ht="14.25" customHeight="1"/>
-    <row r="811" ht="14.25" customHeight="1"/>
-    <row r="812" ht="14.25" customHeight="1"/>
-    <row r="813" ht="14.25" customHeight="1"/>
-    <row r="814" ht="14.25" customHeight="1"/>
-    <row r="815" ht="14.25" customHeight="1"/>
-    <row r="816" ht="14.25" customHeight="1"/>
-    <row r="817" ht="14.25" customHeight="1"/>
-    <row r="818" ht="14.25" customHeight="1"/>
-    <row r="819" ht="14.25" customHeight="1"/>
-    <row r="820" ht="14.25" customHeight="1"/>
-    <row r="821" ht="14.25" customHeight="1"/>
-    <row r="822" ht="14.25" customHeight="1"/>
-    <row r="823" ht="14.25" customHeight="1"/>
-    <row r="824" ht="14.25" customHeight="1"/>
-    <row r="825" ht="14.25" customHeight="1"/>
-    <row r="826" ht="14.25" customHeight="1"/>
-    <row r="827" ht="14.25" customHeight="1"/>
-    <row r="828" ht="14.25" customHeight="1"/>
-    <row r="829" ht="14.25" customHeight="1"/>
-    <row r="830" ht="14.25" customHeight="1"/>
-    <row r="831" ht="14.25" customHeight="1"/>
-    <row r="832" ht="14.25" customHeight="1"/>
-    <row r="833" ht="14.25" customHeight="1"/>
-    <row r="834" ht="14.25" customHeight="1"/>
-    <row r="835" ht="14.25" customHeight="1"/>
-    <row r="836" ht="14.25" customHeight="1"/>
-    <row r="837" ht="14.25" customHeight="1"/>
-    <row r="838" ht="14.25" customHeight="1"/>
-    <row r="839" ht="14.25" customHeight="1"/>
-    <row r="840" ht="14.25" customHeight="1"/>
-    <row r="841" ht="14.25" customHeight="1"/>
-    <row r="842" ht="14.25" customHeight="1"/>
-    <row r="843" ht="14.25" customHeight="1"/>
-    <row r="844" ht="14.25" customHeight="1"/>
-    <row r="845" ht="14.25" customHeight="1"/>
-    <row r="846" ht="14.25" customHeight="1"/>
-    <row r="847" ht="14.25" customHeight="1"/>
-    <row r="848" ht="14.25" customHeight="1"/>
-    <row r="849" ht="14.25" customHeight="1"/>
-    <row r="850" ht="14.25" customHeight="1"/>
-    <row r="851" ht="14.25" customHeight="1"/>
-    <row r="852" ht="14.25" customHeight="1"/>
-    <row r="853" ht="14.25" customHeight="1"/>
-    <row r="854" ht="14.25" customHeight="1"/>
-    <row r="855" ht="14.25" customHeight="1"/>
-    <row r="856" ht="14.25" customHeight="1"/>
-    <row r="857" ht="14.25" customHeight="1"/>
-    <row r="858" ht="14.25" customHeight="1"/>
-    <row r="859" ht="14.25" customHeight="1"/>
-    <row r="860" ht="14.25" customHeight="1"/>
-    <row r="861" ht="14.25" customHeight="1"/>
-    <row r="862" ht="14.25" customHeight="1"/>
-    <row r="863" ht="14.25" customHeight="1"/>
-    <row r="864" ht="14.25" customHeight="1"/>
-    <row r="865" ht="14.25" customHeight="1"/>
-    <row r="866" ht="14.25" customHeight="1"/>
-    <row r="867" ht="14.25" customHeight="1"/>
-    <row r="868" ht="14.25" customHeight="1"/>
-    <row r="869" ht="14.25" customHeight="1"/>
-    <row r="870" ht="14.25" customHeight="1"/>
-    <row r="871" ht="14.25" customHeight="1"/>
-    <row r="872" ht="14.25" customHeight="1"/>
-    <row r="873" ht="14.25" customHeight="1"/>
-    <row r="874" ht="14.25" customHeight="1"/>
-    <row r="875" ht="14.25" customHeight="1"/>
-    <row r="876" ht="14.25" customHeight="1"/>
-    <row r="877" ht="14.25" customHeight="1"/>
-    <row r="878" ht="14.25" customHeight="1"/>
-    <row r="879" ht="14.25" customHeight="1"/>
-    <row r="880" ht="14.25" customHeight="1"/>
-    <row r="881" ht="14.25" customHeight="1"/>
-    <row r="882" ht="14.25" customHeight="1"/>
-    <row r="883" ht="14.25" customHeight="1"/>
-    <row r="884" ht="14.25" customHeight="1"/>
-    <row r="885" ht="14.25" customHeight="1"/>
-    <row r="886" ht="14.25" customHeight="1"/>
-    <row r="887" ht="14.25" customHeight="1"/>
-    <row r="888" ht="14.25" customHeight="1"/>
-    <row r="889" ht="14.25" customHeight="1"/>
-    <row r="890" ht="14.25" customHeight="1"/>
-    <row r="891" ht="14.25" customHeight="1"/>
-    <row r="892" ht="14.25" customHeight="1"/>
-    <row r="893" ht="14.25" customHeight="1"/>
-    <row r="894" ht="14.25" customHeight="1"/>
-    <row r="895" ht="14.25" customHeight="1"/>
-    <row r="896" ht="14.25" customHeight="1"/>
-    <row r="897" ht="14.25" customHeight="1"/>
-    <row r="898" ht="14.25" customHeight="1"/>
-    <row r="899" ht="14.25" customHeight="1"/>
-    <row r="900" ht="14.25" customHeight="1"/>
-    <row r="901" ht="14.25" customHeight="1"/>
-    <row r="902" ht="14.25" customHeight="1"/>
-    <row r="903" ht="14.25" customHeight="1"/>
-    <row r="904" ht="14.25" customHeight="1"/>
-    <row r="905" ht="14.25" customHeight="1"/>
-    <row r="906" ht="14.25" customHeight="1"/>
-    <row r="907" ht="14.25" customHeight="1"/>
-    <row r="908" ht="14.25" customHeight="1"/>
-    <row r="909" ht="14.25" customHeight="1"/>
-    <row r="910" ht="14.25" customHeight="1"/>
-    <row r="911" ht="14.25" customHeight="1"/>
-    <row r="912" ht="14.25" customHeight="1"/>
-    <row r="913" ht="14.25" customHeight="1"/>
-    <row r="914" ht="14.25" customHeight="1"/>
-    <row r="915" ht="14.25" customHeight="1"/>
-    <row r="916" ht="14.25" customHeight="1"/>
-    <row r="917" ht="14.25" customHeight="1"/>
-    <row r="918" ht="14.25" customHeight="1"/>
-    <row r="919" ht="14.25" customHeight="1"/>
-    <row r="920" ht="14.25" customHeight="1"/>
-    <row r="921" ht="14.25" customHeight="1"/>
-    <row r="922" ht="14.25" customHeight="1"/>
-    <row r="923" ht="14.25" customHeight="1"/>
-    <row r="924" ht="14.25" customHeight="1"/>
-    <row r="925" ht="14.25" customHeight="1"/>
-    <row r="926" ht="14.25" customHeight="1"/>
-    <row r="927" ht="14.25" customHeight="1"/>
-    <row r="928" ht="14.25" customHeight="1"/>
-    <row r="929" ht="14.25" customHeight="1"/>
-    <row r="930" ht="14.25" customHeight="1"/>
-    <row r="931" ht="14.25" customHeight="1"/>
-    <row r="932" ht="14.25" customHeight="1"/>
-    <row r="933" ht="14.25" customHeight="1"/>
-    <row r="934" ht="14.25" customHeight="1"/>
-    <row r="935" ht="14.25" customHeight="1"/>
-    <row r="936" ht="14.25" customHeight="1"/>
-    <row r="937" ht="14.25" customHeight="1"/>
-    <row r="938" ht="14.25" customHeight="1"/>
-    <row r="939" ht="14.25" customHeight="1"/>
-    <row r="940" ht="14.25" customHeight="1"/>
-    <row r="941" ht="14.25" customHeight="1"/>
-    <row r="942" ht="14.25" customHeight="1"/>
-    <row r="943" ht="14.25" customHeight="1"/>
-    <row r="944" ht="14.25" customHeight="1"/>
-    <row r="945" ht="14.25" customHeight="1"/>
-    <row r="946" ht="14.25" customHeight="1"/>
-    <row r="947" ht="14.25" customHeight="1"/>
-    <row r="948" ht="14.25" customHeight="1"/>
-    <row r="949" ht="14.25" customHeight="1"/>
-    <row r="950" ht="14.25" customHeight="1"/>
-    <row r="951" ht="14.25" customHeight="1"/>
-    <row r="952" ht="14.25" customHeight="1"/>
-    <row r="953" ht="14.25" customHeight="1"/>
-    <row r="954" ht="14.25" customHeight="1"/>
-    <row r="955" ht="14.25" customHeight="1"/>
-    <row r="956" ht="14.25" customHeight="1"/>
-    <row r="957" ht="14.25" customHeight="1"/>
-    <row r="958" ht="14.25" customHeight="1"/>
-    <row r="959" ht="14.25" customHeight="1"/>
-    <row r="960" ht="14.25" customHeight="1"/>
-    <row r="961" ht="14.25" customHeight="1"/>
-    <row r="962" ht="14.25" customHeight="1"/>
-    <row r="963" ht="14.25" customHeight="1"/>
-    <row r="964" ht="14.25" customHeight="1"/>
-    <row r="965" ht="14.25" customHeight="1"/>
-    <row r="966" ht="14.25" customHeight="1"/>
-    <row r="967" ht="14.25" customHeight="1"/>
-    <row r="968" ht="14.25" customHeight="1"/>
-    <row r="969" ht="14.25" customHeight="1"/>
-    <row r="970" ht="14.25" customHeight="1"/>
-    <row r="971" ht="14.25" customHeight="1"/>
-    <row r="972" ht="14.25" customHeight="1"/>
-    <row r="973" ht="14.25" customHeight="1"/>
-    <row r="974" ht="14.25" customHeight="1"/>
-    <row r="975" ht="14.25" customHeight="1"/>
-    <row r="976" ht="14.25" customHeight="1"/>
-    <row r="977" ht="14.25" customHeight="1"/>
-    <row r="978" ht="14.25" customHeight="1"/>
-    <row r="979" ht="14.25" customHeight="1"/>
-    <row r="980" ht="14.25" customHeight="1"/>
-    <row r="981" ht="14.25" customHeight="1"/>
-    <row r="982" ht="14.25" customHeight="1"/>
-    <row r="983" ht="14.25" customHeight="1"/>
-    <row r="984" ht="14.25" customHeight="1"/>
-    <row r="985" ht="14.25" customHeight="1"/>
-    <row r="986" ht="14.25" customHeight="1"/>
-    <row r="987" ht="14.25" customHeight="1"/>
-    <row r="988" ht="14.25" customHeight="1"/>
-    <row r="989" ht="14.25" customHeight="1"/>
-    <row r="990" ht="14.25" customHeight="1"/>
-    <row r="991" ht="14.25" customHeight="1"/>
-    <row r="992" ht="14.25" customHeight="1"/>
-    <row r="993" ht="14.25" customHeight="1"/>
-    <row r="994" ht="14.25" customHeight="1"/>
-    <row r="995" ht="14.25" customHeight="1"/>
-    <row r="996" ht="14.25" customHeight="1"/>
-    <row r="997" ht="14.25" customHeight="1"/>
-    <row r="998" ht="14.25" customHeight="1"/>
-    <row r="999" ht="14.25" customHeight="1"/>
-    <row r="1000" ht="14.25" customHeight="1"/>
+    <row r="221" ht="15.75" customHeight="1"/>
+    <row r="222" ht="15.75" customHeight="1"/>
+    <row r="223" ht="15.75" customHeight="1"/>
+    <row r="224" ht="15.75" customHeight="1"/>
+    <row r="225" ht="15.75" customHeight="1"/>
+    <row r="226" ht="15.75" customHeight="1"/>
+    <row r="227" ht="15.75" customHeight="1"/>
+    <row r="228" ht="15.75" customHeight="1"/>
+    <row r="229" ht="15.75" customHeight="1"/>
+    <row r="230" ht="15.75" customHeight="1"/>
+    <row r="231" ht="15.75" customHeight="1"/>
+    <row r="232" ht="15.75" customHeight="1"/>
+    <row r="233" ht="15.75" customHeight="1"/>
+    <row r="234" ht="15.75" customHeight="1"/>
+    <row r="235" ht="15.75" customHeight="1"/>
+    <row r="236" ht="15.75" customHeight="1"/>
+    <row r="237" ht="15.75" customHeight="1"/>
+    <row r="238" ht="15.75" customHeight="1"/>
+    <row r="239" ht="15.75" customHeight="1"/>
+    <row r="240" ht="15.75" customHeight="1"/>
+    <row r="241" ht="15.75" customHeight="1"/>
+    <row r="242" ht="15.75" customHeight="1"/>
+    <row r="243" ht="15.75" customHeight="1"/>
+    <row r="244" ht="15.75" customHeight="1"/>
+    <row r="245" ht="15.75" customHeight="1"/>
+    <row r="246" ht="15.75" customHeight="1"/>
+    <row r="247" ht="15.75" customHeight="1"/>
+    <row r="248" ht="15.75" customHeight="1"/>
+    <row r="249" ht="15.75" customHeight="1"/>
+    <row r="250" ht="15.75" customHeight="1"/>
+    <row r="251" ht="15.75" customHeight="1"/>
+    <row r="252" ht="15.75" customHeight="1"/>
+    <row r="253" ht="15.75" customHeight="1"/>
+    <row r="254" ht="15.75" customHeight="1"/>
+    <row r="255" ht="15.75" customHeight="1"/>
+    <row r="256" ht="15.75" customHeight="1"/>
+    <row r="257" ht="15.75" customHeight="1"/>
+    <row r="258" ht="15.75" customHeight="1"/>
+    <row r="259" ht="15.75" customHeight="1"/>
+    <row r="260" ht="15.75" customHeight="1"/>
+    <row r="261" ht="15.75" customHeight="1"/>
+    <row r="262" ht="15.75" customHeight="1"/>
+    <row r="263" ht="15.75" customHeight="1"/>
+    <row r="264" ht="15.75" customHeight="1"/>
+    <row r="265" ht="15.75" customHeight="1"/>
+    <row r="266" ht="15.75" customHeight="1"/>
+    <row r="267" ht="15.75" customHeight="1"/>
+    <row r="268" ht="15.75" customHeight="1"/>
+    <row r="269" ht="15.75" customHeight="1"/>
+    <row r="270" ht="15.75" customHeight="1"/>
+    <row r="271" ht="15.75" customHeight="1"/>
+    <row r="272" ht="15.75" customHeight="1"/>
+    <row r="273" ht="15.75" customHeight="1"/>
+    <row r="274" ht="15.75" customHeight="1"/>
+    <row r="275" ht="15.75" customHeight="1"/>
+    <row r="276" ht="15.75" customHeight="1"/>
+    <row r="277" ht="15.75" customHeight="1"/>
+    <row r="278" ht="15.75" customHeight="1"/>
+    <row r="279" ht="15.75" customHeight="1"/>
+    <row r="280" ht="15.75" customHeight="1"/>
+    <row r="281" ht="15.75" customHeight="1"/>
+    <row r="282" ht="15.75" customHeight="1"/>
+    <row r="283" ht="15.75" customHeight="1"/>
+    <row r="284" ht="15.75" customHeight="1"/>
+    <row r="285" ht="15.75" customHeight="1"/>
+    <row r="286" ht="15.75" customHeight="1"/>
+    <row r="287" ht="15.75" customHeight="1"/>
+    <row r="288" ht="15.75" customHeight="1"/>
+    <row r="289" ht="15.75" customHeight="1"/>
+    <row r="290" ht="15.75" customHeight="1"/>
+    <row r="291" ht="15.75" customHeight="1"/>
+    <row r="292" ht="15.75" customHeight="1"/>
+    <row r="293" ht="15.75" customHeight="1"/>
+    <row r="294" ht="15.75" customHeight="1"/>
+    <row r="295" ht="15.75" customHeight="1"/>
+    <row r="296" ht="15.75" customHeight="1"/>
+    <row r="297" ht="15.75" customHeight="1"/>
+    <row r="298" ht="15.75" customHeight="1"/>
+    <row r="299" ht="15.75" customHeight="1"/>
+    <row r="300" ht="15.75" customHeight="1"/>
+    <row r="301" ht="15.75" customHeight="1"/>
+    <row r="302" ht="15.75" customHeight="1"/>
+    <row r="303" ht="15.75" customHeight="1"/>
+    <row r="304" ht="15.75" customHeight="1"/>
+    <row r="305" ht="15.75" customHeight="1"/>
+    <row r="306" ht="15.75" customHeight="1"/>
+    <row r="307" ht="15.75" customHeight="1"/>
+    <row r="308" ht="15.75" customHeight="1"/>
+    <row r="309" ht="15.75" customHeight="1"/>
+    <row r="310" ht="15.75" customHeight="1"/>
+    <row r="311" ht="15.75" customHeight="1"/>
+    <row r="312" ht="15.75" customHeight="1"/>
+    <row r="313" ht="15.75" customHeight="1"/>
+    <row r="314" ht="15.75" customHeight="1"/>
+    <row r="315" ht="15.75" customHeight="1"/>
+    <row r="316" ht="15.75" customHeight="1"/>
+    <row r="317" ht="15.75" customHeight="1"/>
+    <row r="318" ht="15.75" customHeight="1"/>
+    <row r="319" ht="15.75" customHeight="1"/>
+    <row r="320" ht="15.75" customHeight="1"/>
+    <row r="321" ht="15.75" customHeight="1"/>
+    <row r="322" ht="15.75" customHeight="1"/>
+    <row r="323" ht="15.75" customHeight="1"/>
+    <row r="324" ht="15.75" customHeight="1"/>
+    <row r="325" ht="15.75" customHeight="1"/>
+    <row r="326" ht="15.75" customHeight="1"/>
+    <row r="327" ht="15.75" customHeight="1"/>
+    <row r="328" ht="15.75" customHeight="1"/>
+    <row r="329" ht="15.75" customHeight="1"/>
+    <row r="330" ht="15.75" customHeight="1"/>
+    <row r="331" ht="15.75" customHeight="1"/>
+    <row r="332" ht="15.75" customHeight="1"/>
+    <row r="333" ht="15.75" customHeight="1"/>
+    <row r="334" ht="15.75" customHeight="1"/>
+    <row r="335" ht="15.75" customHeight="1"/>
+    <row r="336" ht="15.75" customHeight="1"/>
+    <row r="337" ht="15.75" customHeight="1"/>
+    <row r="338" ht="15.75" customHeight="1"/>
+    <row r="339" ht="15.75" customHeight="1"/>
+    <row r="340" ht="15.75" customHeight="1"/>
+    <row r="341" ht="15.75" customHeight="1"/>
+    <row r="342" ht="15.75" customHeight="1"/>
+    <row r="343" ht="15.75" customHeight="1"/>
+    <row r="344" ht="15.75" customHeight="1"/>
+    <row r="345" ht="15.75" customHeight="1"/>
+    <row r="346" ht="15.75" customHeight="1"/>
+    <row r="347" ht="15.75" customHeight="1"/>
+    <row r="348" ht="15.75" customHeight="1"/>
+    <row r="349" ht="15.75" customHeight="1"/>
+    <row r="350" ht="15.75" customHeight="1"/>
+    <row r="351" ht="15.75" customHeight="1"/>
+    <row r="352" ht="15.75" customHeight="1"/>
+    <row r="353" ht="15.75" customHeight="1"/>
+    <row r="354" ht="15.75" customHeight="1"/>
+    <row r="355" ht="15.75" customHeight="1"/>
+    <row r="356" ht="15.75" customHeight="1"/>
+    <row r="357" ht="15.75" customHeight="1"/>
+    <row r="358" ht="15.75" customHeight="1"/>
+    <row r="359" ht="15.75" customHeight="1"/>
+    <row r="360" ht="15.75" customHeight="1"/>
+    <row r="361" ht="15.75" customHeight="1"/>
+    <row r="362" ht="15.75" customHeight="1"/>
+    <row r="363" ht="15.75" customHeight="1"/>
+    <row r="364" ht="15.75" customHeight="1"/>
+    <row r="365" ht="15.75" customHeight="1"/>
+    <row r="366" ht="15.75" customHeight="1"/>
+    <row r="367" ht="15.75" customHeight="1"/>
+    <row r="368" ht="15.75" customHeight="1"/>
+    <row r="369" ht="15.75" customHeight="1"/>
+    <row r="370" ht="15.75" customHeight="1"/>
+    <row r="371" ht="15.75" customHeight="1"/>
+    <row r="372" ht="15.75" customHeight="1"/>
+    <row r="373" ht="15.75" customHeight="1"/>
+    <row r="374" ht="15.75" customHeight="1"/>
+    <row r="375" ht="15.75" customHeight="1"/>
+    <row r="376" ht="15.75" customHeight="1"/>
+    <row r="377" ht="15.75" customHeight="1"/>
+    <row r="378" ht="15.75" customHeight="1"/>
+    <row r="379" ht="15.75" customHeight="1"/>
+    <row r="380" ht="15.75" customHeight="1"/>
+    <row r="381" ht="15.75" customHeight="1"/>
+    <row r="382" ht="15.75" customHeight="1"/>
+    <row r="383" ht="15.75" customHeight="1"/>
+    <row r="384" ht="15.75" customHeight="1"/>
+    <row r="385" ht="15.75" customHeight="1"/>
+    <row r="386" ht="15.75" customHeight="1"/>
+    <row r="387" ht="15.75" customHeight="1"/>
+    <row r="388" ht="15.75" customHeight="1"/>
+    <row r="389" ht="15.75" customHeight="1"/>
+    <row r="390" ht="15.75" customHeight="1"/>
+    <row r="391" ht="15.75" customHeight="1"/>
+    <row r="392" ht="15.75" customHeight="1"/>
+    <row r="393" ht="15.75" customHeight="1"/>
+    <row r="394" ht="15.75" customHeight="1"/>
+    <row r="395" ht="15.75" customHeight="1"/>
+    <row r="396" ht="15.75" customHeight="1"/>
+    <row r="397" ht="15.75" customHeight="1"/>
+    <row r="398" ht="15.75" customHeight="1"/>
+    <row r="399" ht="15.75" customHeight="1"/>
+    <row r="400" ht="15.75" customHeight="1"/>
+    <row r="401" ht="15.75" customHeight="1"/>
+    <row r="402" ht="15.75" customHeight="1"/>
+    <row r="403" ht="15.75" customHeight="1"/>
+    <row r="404" ht="15.75" customHeight="1"/>
+    <row r="405" ht="15.75" customHeight="1"/>
+    <row r="406" ht="15.75" customHeight="1"/>
+    <row r="407" ht="15.75" customHeight="1"/>
+    <row r="408" ht="15.75" customHeight="1"/>
+    <row r="409" ht="15.75" customHeight="1"/>
+    <row r="410" ht="15.75" customHeight="1"/>
+    <row r="411" ht="15.75" customHeight="1"/>
+    <row r="412" ht="15.75" customHeight="1"/>
+    <row r="413" ht="15.75" customHeight="1"/>
+    <row r="414" ht="15.75" customHeight="1"/>
+    <row r="415" ht="15.75" customHeight="1"/>
+    <row r="416" ht="15.75" customHeight="1"/>
+    <row r="417" ht="15.75" customHeight="1"/>
+    <row r="418" ht="15.75" customHeight="1"/>
+    <row r="419" ht="15.75" customHeight="1"/>
+    <row r="420" ht="15.75" customHeight="1"/>
+    <row r="421" ht="15.75" customHeight="1"/>
+    <row r="422" ht="15.75" customHeight="1"/>
+    <row r="423" ht="15.75" customHeight="1"/>
+    <row r="424" ht="15.75" customHeight="1"/>
+    <row r="425" ht="15.75" customHeight="1"/>
+    <row r="426" ht="15.75" customHeight="1"/>
+    <row r="427" ht="15.75" customHeight="1"/>
+    <row r="428" ht="15.75" customHeight="1"/>
+    <row r="429" ht="15.75" customHeight="1"/>
+    <row r="430" ht="15.75" customHeight="1"/>
+    <row r="431" ht="15.75" customHeight="1"/>
+    <row r="432" ht="15.75" customHeight="1"/>
+    <row r="433" ht="15.75" customHeight="1"/>
+    <row r="434" ht="15.75" customHeight="1"/>
+    <row r="435" ht="15.75" customHeight="1"/>
+    <row r="436" ht="15.75" customHeight="1"/>
+    <row r="437" ht="15.75" customHeight="1"/>
+    <row r="438" ht="15.75" customHeight="1"/>
+    <row r="439" ht="15.75" customHeight="1"/>
+    <row r="440" ht="15.75" customHeight="1"/>
+    <row r="441" ht="15.75" customHeight="1"/>
+    <row r="442" ht="15.75" customHeight="1"/>
+    <row r="443" ht="15.75" customHeight="1"/>
+    <row r="444" ht="15.75" customHeight="1"/>
+    <row r="445" ht="15.75" customHeight="1"/>
+    <row r="446" ht="15.75" customHeight="1"/>
+    <row r="447" ht="15.75" customHeight="1"/>
+    <row r="448" ht="15.75" customHeight="1"/>
+    <row r="449" ht="15.75" customHeight="1"/>
+    <row r="450" ht="15.75" customHeight="1"/>
+    <row r="451" ht="15.75" customHeight="1"/>
+    <row r="452" ht="15.75" customHeight="1"/>
+    <row r="453" ht="15.75" customHeight="1"/>
+    <row r="454" ht="15.75" customHeight="1"/>
+    <row r="455" ht="15.75" customHeight="1"/>
+    <row r="456" ht="15.75" customHeight="1"/>
+    <row r="457" ht="15.75" customHeight="1"/>
+    <row r="458" ht="15.75" customHeight="1"/>
+    <row r="459" ht="15.75" customHeight="1"/>
+    <row r="460" ht="15.75" customHeight="1"/>
+    <row r="461" ht="15.75" customHeight="1"/>
+    <row r="462" ht="15.75" customHeight="1"/>
+    <row r="463" ht="15.75" customHeight="1"/>
+    <row r="464" ht="15.75" customHeight="1"/>
+    <row r="465" ht="15.75" customHeight="1"/>
+    <row r="466" ht="15.75" customHeight="1"/>
+    <row r="467" ht="15.75" customHeight="1"/>
+    <row r="468" ht="15.75" customHeight="1"/>
+    <row r="469" ht="15.75" customHeight="1"/>
+    <row r="470" ht="15.75" customHeight="1"/>
+    <row r="471" ht="15.75" customHeight="1"/>
+    <row r="472" ht="15.75" customHeight="1"/>
+    <row r="473" ht="15.75" customHeight="1"/>
+    <row r="474" ht="15.75" customHeight="1"/>
+    <row r="475" ht="15.75" customHeight="1"/>
+    <row r="476" ht="15.75" customHeight="1"/>
+    <row r="477" ht="15.75" customHeight="1"/>
+    <row r="478" ht="15.75" customHeight="1"/>
+    <row r="479" ht="15.75" customHeight="1"/>
+    <row r="480" ht="15.75" customHeight="1"/>
+    <row r="481" ht="15.75" customHeight="1"/>
+    <row r="482" ht="15.75" customHeight="1"/>
+    <row r="483" ht="15.75" customHeight="1"/>
+    <row r="484" ht="15.75" customHeight="1"/>
+    <row r="485" ht="15.75" customHeight="1"/>
+    <row r="486" ht="15.75" customHeight="1"/>
+    <row r="487" ht="15.75" customHeight="1"/>
+    <row r="488" ht="15.75" customHeight="1"/>
+    <row r="489" ht="15.75" customHeight="1"/>
+    <row r="490" ht="15.75" customHeight="1"/>
+    <row r="491" ht="15.75" customHeight="1"/>
+    <row r="492" ht="15.75" customHeight="1"/>
+    <row r="493" ht="15.75" customHeight="1"/>
+    <row r="494" ht="15.75" customHeight="1"/>
+    <row r="495" ht="15.75" customHeight="1"/>
+    <row r="496" ht="15.75" customHeight="1"/>
+    <row r="497" ht="15.75" customHeight="1"/>
+    <row r="498" ht="15.75" customHeight="1"/>
+    <row r="499" ht="15.75" customHeight="1"/>
+    <row r="500" ht="15.75" customHeight="1"/>
+    <row r="501" ht="15.75" customHeight="1"/>
+    <row r="502" ht="15.75" customHeight="1"/>
+    <row r="503" ht="15.75" customHeight="1"/>
+    <row r="504" ht="15.75" customHeight="1"/>
+    <row r="505" ht="15.75" customHeight="1"/>
+    <row r="506" ht="15.75" customHeight="1"/>
+    <row r="507" ht="15.75" customHeight="1"/>
+    <row r="508" ht="15.75" customHeight="1"/>
+    <row r="509" ht="15.75" customHeight="1"/>
+    <row r="510" ht="15.75" customHeight="1"/>
+    <row r="511" ht="15.75" customHeight="1"/>
+    <row r="512" ht="15.75" customHeight="1"/>
+    <row r="513" ht="15.75" customHeight="1"/>
+    <row r="514" ht="15.75" customHeight="1"/>
+    <row r="515" ht="15.75" customHeight="1"/>
+    <row r="516" ht="15.75" customHeight="1"/>
+    <row r="517" ht="15.75" customHeight="1"/>
+    <row r="518" ht="15.75" customHeight="1"/>
+    <row r="519" ht="15.75" customHeight="1"/>
+    <row r="520" ht="15.75" customHeight="1"/>
+    <row r="521" ht="15.75" customHeight="1"/>
+    <row r="522" ht="15.75" customHeight="1"/>
+    <row r="523" ht="15.75" customHeight="1"/>
+    <row r="524" ht="15.75" customHeight="1"/>
+    <row r="525" ht="15.75" customHeight="1"/>
+    <row r="526" ht="15.75" customHeight="1"/>
+    <row r="527" ht="15.75" customHeight="1"/>
+    <row r="528" ht="15.75" customHeight="1"/>
+    <row r="529" ht="15.75" customHeight="1"/>
+    <row r="530" ht="15.75" customHeight="1"/>
+    <row r="531" ht="15.75" customHeight="1"/>
+    <row r="532" ht="15.75" customHeight="1"/>
+    <row r="533" ht="15.75" customHeight="1"/>
+    <row r="534" ht="15.75" customHeight="1"/>
+    <row r="535" ht="15.75" customHeight="1"/>
+    <row r="536" ht="15.75" customHeight="1"/>
+    <row r="537" ht="15.75" customHeight="1"/>
+    <row r="538" ht="15.75" customHeight="1"/>
+    <row r="539" ht="15.75" customHeight="1"/>
+    <row r="540" ht="15.75" customHeight="1"/>
+    <row r="541" ht="15.75" customHeight="1"/>
+    <row r="542" ht="15.75" customHeight="1"/>
+    <row r="543" ht="15.75" customHeight="1"/>
+    <row r="544" ht="15.75" customHeight="1"/>
+    <row r="545" ht="15.75" customHeight="1"/>
+    <row r="546" ht="15.75" customHeight="1"/>
+    <row r="547" ht="15.75" customHeight="1"/>
+    <row r="548" ht="15.75" customHeight="1"/>
+    <row r="549" ht="15.75" customHeight="1"/>
+    <row r="550" ht="15.75" customHeight="1"/>
+    <row r="551" ht="15.75" customHeight="1"/>
+    <row r="552" ht="15.75" customHeight="1"/>
+    <row r="553" ht="15.75" customHeight="1"/>
+    <row r="554" ht="15.75" customHeight="1"/>
+    <row r="555" ht="15.75" customHeight="1"/>
+    <row r="556" ht="15.75" customHeight="1"/>
+    <row r="557" ht="15.75" customHeight="1"/>
+    <row r="558" ht="15.75" customHeight="1"/>
+    <row r="559" ht="15.75" customHeight="1"/>
+    <row r="560" ht="15.75" customHeight="1"/>
+    <row r="561" ht="15.75" customHeight="1"/>
+    <row r="562" ht="15.75" customHeight="1"/>
+    <row r="563" ht="15.75" customHeight="1"/>
+    <row r="564" ht="15.75" customHeight="1"/>
+    <row r="565" ht="15.75" customHeight="1"/>
+    <row r="566" ht="15.75" customHeight="1"/>
+    <row r="567" ht="15.75" customHeight="1"/>
+    <row r="568" ht="15.75" customHeight="1"/>
+    <row r="569" ht="15.75" customHeight="1"/>
+    <row r="570" ht="15.75" customHeight="1"/>
+    <row r="571" ht="15.75" customHeight="1"/>
+    <row r="572" ht="15.75" customHeight="1"/>
+    <row r="573" ht="15.75" customHeight="1"/>
+    <row r="574" ht="15.75" customHeight="1"/>
+    <row r="575" ht="15.75" customHeight="1"/>
+    <row r="576" ht="15.75" customHeight="1"/>
+    <row r="577" ht="15.75" customHeight="1"/>
+    <row r="578" ht="15.75" customHeight="1"/>
+    <row r="579" ht="15.75" customHeight="1"/>
+    <row r="580" ht="15.75" customHeight="1"/>
+    <row r="581" ht="15.75" customHeight="1"/>
+    <row r="582" ht="15.75" customHeight="1"/>
+    <row r="583" ht="15.75" customHeight="1"/>
+    <row r="584" ht="15.75" customHeight="1"/>
+    <row r="585" ht="15.75" customHeight="1"/>
+    <row r="586" ht="15.75" customHeight="1"/>
+    <row r="587" ht="15.75" customHeight="1"/>
+    <row r="588" ht="15.75" customHeight="1"/>
+    <row r="589" ht="15.75" customHeight="1"/>
+    <row r="590" ht="15.75" customHeight="1"/>
+    <row r="591" ht="15.75" customHeight="1"/>
+    <row r="592" ht="15.75" customHeight="1"/>
+    <row r="593" ht="15.75" customHeight="1"/>
+    <row r="594" ht="15.75" customHeight="1"/>
+    <row r="595" ht="15.75" customHeight="1"/>
+    <row r="596" ht="15.75" customHeight="1"/>
+    <row r="597" ht="15.75" customHeight="1"/>
+    <row r="598" ht="15.75" customHeight="1"/>
+    <row r="599" ht="15.75" customHeight="1"/>
+    <row r="600" ht="15.75" customHeight="1"/>
+    <row r="601" ht="15.75" customHeight="1"/>
+    <row r="602" ht="15.75" customHeight="1"/>
+    <row r="603" ht="15.75" customHeight="1"/>
+    <row r="604" ht="15.75" customHeight="1"/>
+    <row r="605" ht="15.75" customHeight="1"/>
+    <row r="606" ht="15.75" customHeight="1"/>
+    <row r="607" ht="15.75" customHeight="1"/>
+    <row r="608" ht="15.75" customHeight="1"/>
+    <row r="609" ht="15.75" customHeight="1"/>
+    <row r="610" ht="15.75" customHeight="1"/>
+    <row r="611" ht="15.75" customHeight="1"/>
+    <row r="612" ht="15.75" customHeight="1"/>
+    <row r="613" ht="15.75" customHeight="1"/>
+    <row r="614" ht="15.75" customHeight="1"/>
+    <row r="615" ht="15.75" customHeight="1"/>
+    <row r="616" ht="15.75" customHeight="1"/>
+    <row r="617" ht="15.75" customHeight="1"/>
+    <row r="618" ht="15.75" customHeight="1"/>
+    <row r="619" ht="15.75" customHeight="1"/>
+    <row r="620" ht="15.75" customHeight="1"/>
+    <row r="621" ht="15.75" customHeight="1"/>
+    <row r="622" ht="15.75" customHeight="1"/>
+    <row r="623" ht="15.75" customHeight="1"/>
+    <row r="624" ht="15.75" customHeight="1"/>
+    <row r="625" ht="15.75" customHeight="1"/>
+    <row r="626" ht="15.75" customHeight="1"/>
+    <row r="627" ht="15.75" customHeight="1"/>
+    <row r="628" ht="15.75" customHeight="1"/>
+    <row r="629" ht="15.75" customHeight="1"/>
+    <row r="630" ht="15.75" customHeight="1"/>
+    <row r="631" ht="15.75" customHeight="1"/>
+    <row r="632" ht="15.75" customHeight="1"/>
+    <row r="633" ht="15.75" customHeight="1"/>
+    <row r="634" ht="15.75" customHeight="1"/>
+    <row r="635" ht="15.75" customHeight="1"/>
+    <row r="636" ht="15.75" customHeight="1"/>
+    <row r="637" ht="15.75" customHeight="1"/>
+    <row r="638" ht="15.75" customHeight="1"/>
+    <row r="639" ht="15.75" customHeight="1"/>
+    <row r="640" ht="15.75" customHeight="1"/>
+    <row r="641" ht="15.75" customHeight="1"/>
+    <row r="642" ht="15.75" customHeight="1"/>
+    <row r="643" ht="15.75" customHeight="1"/>
+    <row r="644" ht="15.75" customHeight="1"/>
+    <row r="645" ht="15.75" customHeight="1"/>
+    <row r="646" ht="15.75" customHeight="1"/>
+    <row r="647" ht="15.75" customHeight="1"/>
+    <row r="648" ht="15.75" customHeight="1"/>
+    <row r="649" ht="15.75" customHeight="1"/>
+    <row r="650" ht="15.75" customHeight="1"/>
+    <row r="651" ht="15.75" customHeight="1"/>
+    <row r="652" ht="15.75" customHeight="1"/>
+    <row r="653" ht="15.75" customHeight="1"/>
+    <row r="654" ht="15.75" customHeight="1"/>
+    <row r="655" ht="15.75" customHeight="1"/>
+    <row r="656" ht="15.75" customHeight="1"/>
+    <row r="657" ht="15.75" customHeight="1"/>
+    <row r="658" ht="15.75" customHeight="1"/>
+    <row r="659" ht="15.75" customHeight="1"/>
+    <row r="660" ht="15.75" customHeight="1"/>
+    <row r="661" ht="15.75" customHeight="1"/>
+    <row r="662" ht="15.75" customHeight="1"/>
+    <row r="663" ht="15.75" customHeight="1"/>
+    <row r="664" ht="15.75" customHeight="1"/>
+    <row r="665" ht="15.75" customHeight="1"/>
+    <row r="666" ht="15.75" customHeight="1"/>
+    <row r="667" ht="15.75" customHeight="1"/>
+    <row r="668" ht="15.75" customHeight="1"/>
+    <row r="669" ht="15.75" customHeight="1"/>
+    <row r="670" ht="15.75" customHeight="1"/>
+    <row r="671" ht="15.75" customHeight="1"/>
+    <row r="672" ht="15.75" customHeight="1"/>
+    <row r="673" ht="15.75" customHeight="1"/>
+    <row r="674" ht="15.75" customHeight="1"/>
+    <row r="675" ht="15.75" customHeight="1"/>
+    <row r="676" ht="15.75" customHeight="1"/>
+    <row r="677" ht="15.75" customHeight="1"/>
+    <row r="678" ht="15.75" customHeight="1"/>
+    <row r="679" ht="15.75" customHeight="1"/>
+    <row r="680" ht="15.75" customHeight="1"/>
+    <row r="681" ht="15.75" customHeight="1"/>
+    <row r="682" ht="15.75" customHeight="1"/>
+    <row r="683" ht="15.75" customHeight="1"/>
+    <row r="684" ht="15.75" customHeight="1"/>
+    <row r="685" ht="15.75" customHeight="1"/>
+    <row r="686" ht="15.75" customHeight="1"/>
+    <row r="687" ht="15.75" customHeight="1"/>
+    <row r="688" ht="15.75" customHeight="1"/>
+    <row r="689" ht="15.75" customHeight="1"/>
+    <row r="690" ht="15.75" customHeight="1"/>
+    <row r="691" ht="15.75" customHeight="1"/>
+    <row r="692" ht="15.75" customHeight="1"/>
+    <row r="693" ht="15.75" customHeight="1"/>
+    <row r="694" ht="15.75" customHeight="1"/>
+    <row r="695" ht="15.75" customHeight="1"/>
+    <row r="696" ht="15.75" customHeight="1"/>
+    <row r="697" ht="15.75" customHeight="1"/>
+    <row r="698" ht="15.75" customHeight="1"/>
+    <row r="699" ht="15.75" customHeight="1"/>
+    <row r="700" ht="15.75" customHeight="1"/>
+    <row r="701" ht="15.75" customHeight="1"/>
+    <row r="702" ht="15.75" customHeight="1"/>
+    <row r="703" ht="15.75" customHeight="1"/>
+    <row r="704" ht="15.75" customHeight="1"/>
+    <row r="705" ht="15.75" customHeight="1"/>
+    <row r="706" ht="15.75" customHeight="1"/>
+    <row r="707" ht="15.75" customHeight="1"/>
+    <row r="708" ht="15.75" customHeight="1"/>
+    <row r="709" ht="15.75" customHeight="1"/>
+    <row r="710" ht="15.75" customHeight="1"/>
+    <row r="711" ht="15.75" customHeight="1"/>
+    <row r="712" ht="15.75" customHeight="1"/>
+    <row r="713" ht="15.75" customHeight="1"/>
+    <row r="714" ht="15.75" customHeight="1"/>
+    <row r="715" ht="15.75" customHeight="1"/>
+    <row r="716" ht="15.75" customHeight="1"/>
+    <row r="717" ht="15.75" customHeight="1"/>
+    <row r="718" ht="15.75" customHeight="1"/>
+    <row r="719" ht="15.75" customHeight="1"/>
+    <row r="720" ht="15.75" customHeight="1"/>
+    <row r="721" ht="15.75" customHeight="1"/>
+    <row r="722" ht="15.75" customHeight="1"/>
+    <row r="723" ht="15.75" customHeight="1"/>
+    <row r="724" ht="15.75" customHeight="1"/>
+    <row r="725" ht="15.75" customHeight="1"/>
+    <row r="726" ht="15.75" customHeight="1"/>
+    <row r="727" ht="15.75" customHeight="1"/>
+    <row r="728" ht="15.75" customHeight="1"/>
+    <row r="729" ht="15.75" customHeight="1"/>
+    <row r="730" ht="15.75" customHeight="1"/>
+    <row r="731" ht="15.75" customHeight="1"/>
+    <row r="732" ht="15.75" customHeight="1"/>
+    <row r="733" ht="15.75" customHeight="1"/>
+    <row r="734" ht="15.75" customHeight="1"/>
+    <row r="735" ht="15.75" customHeight="1"/>
+    <row r="736" ht="15.75" customHeight="1"/>
+    <row r="737" ht="15.75" customHeight="1"/>
+    <row r="738" ht="15.75" customHeight="1"/>
+    <row r="739" ht="15.75" customHeight="1"/>
+    <row r="740" ht="15.75" customHeight="1"/>
+    <row r="741" ht="15.75" customHeight="1"/>
+    <row r="742" ht="15.75" customHeight="1"/>
+    <row r="743" ht="15.75" customHeight="1"/>
+    <row r="744" ht="15.75" customHeight="1"/>
+    <row r="745" ht="15.75" customHeight="1"/>
+    <row r="746" ht="15.75" customHeight="1"/>
+    <row r="747" ht="15.75" customHeight="1"/>
+    <row r="748" ht="15.75" customHeight="1"/>
+    <row r="749" ht="15.75" customHeight="1"/>
+    <row r="750" ht="15.75" customHeight="1"/>
+    <row r="751" ht="15.75" customHeight="1"/>
+    <row r="752" ht="15.75" customHeight="1"/>
+    <row r="753" ht="15.75" customHeight="1"/>
+    <row r="754" ht="15.75" customHeight="1"/>
+    <row r="755" ht="15.75" customHeight="1"/>
+    <row r="756" ht="15.75" customHeight="1"/>
+    <row r="757" ht="15.75" customHeight="1"/>
+    <row r="758" ht="15.75" customHeight="1"/>
+    <row r="759" ht="15.75" customHeight="1"/>
+    <row r="760" ht="15.75" customHeight="1"/>
+    <row r="761" ht="15.75" customHeight="1"/>
+    <row r="762" ht="15.75" customHeight="1"/>
+    <row r="763" ht="15.75" customHeight="1"/>
+    <row r="764" ht="15.75" customHeight="1"/>
+    <row r="765" ht="15.75" customHeight="1"/>
+    <row r="766" ht="15.75" customHeight="1"/>
+    <row r="767" ht="15.75" customHeight="1"/>
+    <row r="768" ht="15.75" customHeight="1"/>
+    <row r="769" ht="15.75" customHeight="1"/>
+    <row r="770" ht="15.75" customHeight="1"/>
+    <row r="771" ht="15.75" customHeight="1"/>
+    <row r="772" ht="15.75" customHeight="1"/>
+    <row r="773" ht="15.75" customHeight="1"/>
+    <row r="774" ht="15.75" customHeight="1"/>
+    <row r="775" ht="15.75" customHeight="1"/>
+    <row r="776" ht="15.75" customHeight="1"/>
+    <row r="777" ht="15.75" customHeight="1"/>
+    <row r="778" ht="15.75" customHeight="1"/>
+    <row r="779" ht="15.75" customHeight="1"/>
+    <row r="780" ht="15.75" customHeight="1"/>
+    <row r="781" ht="15.75" customHeight="1"/>
+    <row r="782" ht="15.75" customHeight="1"/>
+    <row r="783" ht="15.75" customHeight="1"/>
+    <row r="784" ht="15.75" customHeight="1"/>
+    <row r="785" ht="15.75" customHeight="1"/>
+    <row r="786" ht="15.75" customHeight="1"/>
+    <row r="787" ht="15.75" customHeight="1"/>
+    <row r="788" ht="15.75" customHeight="1"/>
+    <row r="789" ht="15.75" customHeight="1"/>
+    <row r="790" ht="15.75" customHeight="1"/>
+    <row r="791" ht="15.75" customHeight="1"/>
+    <row r="792" ht="15.75" customHeight="1"/>
+    <row r="793" ht="15.75" customHeight="1"/>
+    <row r="794" ht="15.75" customHeight="1"/>
+    <row r="795" ht="15.75" customHeight="1"/>
+    <row r="796" ht="15.75" customHeight="1"/>
+    <row r="797" ht="15.75" customHeight="1"/>
+    <row r="798" ht="15.75" customHeight="1"/>
+    <row r="799" ht="15.75" customHeight="1"/>
+    <row r="800" ht="15.75" customHeight="1"/>
+    <row r="801" ht="15.75" customHeight="1"/>
+    <row r="802" ht="15.75" customHeight="1"/>
+    <row r="803" ht="15.75" customHeight="1"/>
+    <row r="804" ht="15.75" customHeight="1"/>
+    <row r="805" ht="15.75" customHeight="1"/>
+    <row r="806" ht="15.75" customHeight="1"/>
+    <row r="807" ht="15.75" customHeight="1"/>
+    <row r="808" ht="15.75" customHeight="1"/>
+    <row r="809" ht="15.75" customHeight="1"/>
+    <row r="810" ht="15.75" customHeight="1"/>
+    <row r="811" ht="15.75" customHeight="1"/>
+    <row r="812" ht="15.75" customHeight="1"/>
+    <row r="813" ht="15.75" customHeight="1"/>
+    <row r="814" ht="15.75" customHeight="1"/>
+    <row r="815" ht="15.75" customHeight="1"/>
+    <row r="816" ht="15.75" customHeight="1"/>
+    <row r="817" ht="15.75" customHeight="1"/>
+    <row r="818" ht="15.75" customHeight="1"/>
+    <row r="819" ht="15.75" customHeight="1"/>
+    <row r="820" ht="15.75" customHeight="1"/>
+    <row r="821" ht="15.75" customHeight="1"/>
+    <row r="822" ht="15.75" customHeight="1"/>
+    <row r="823" ht="15.75" customHeight="1"/>
+    <row r="824" ht="15.75" customHeight="1"/>
+    <row r="825" ht="15.75" customHeight="1"/>
+    <row r="826" ht="15.75" customHeight="1"/>
+    <row r="827" ht="15.75" customHeight="1"/>
+    <row r="828" ht="15.75" customHeight="1"/>
+    <row r="829" ht="15.75" customHeight="1"/>
+    <row r="830" ht="15.75" customHeight="1"/>
+    <row r="831" ht="15.75" customHeight="1"/>
+    <row r="832" ht="15.75" customHeight="1"/>
+    <row r="833" ht="15.75" customHeight="1"/>
+    <row r="834" ht="15.75" customHeight="1"/>
+    <row r="835" ht="15.75" customHeight="1"/>
+    <row r="836" ht="15.75" customHeight="1"/>
+    <row r="837" ht="15.75" customHeight="1"/>
+    <row r="838" ht="15.75" customHeight="1"/>
+    <row r="839" ht="15.75" customHeight="1"/>
+    <row r="840" ht="15.75" customHeight="1"/>
+    <row r="841" ht="15.75" customHeight="1"/>
+    <row r="842" ht="15.75" customHeight="1"/>
+    <row r="843" ht="15.75" customHeight="1"/>
+    <row r="844" ht="15.75" customHeight="1"/>
+    <row r="845" ht="15.75" customHeight="1"/>
+    <row r="846" ht="15.75" customHeight="1"/>
+    <row r="847" ht="15.75" customHeight="1"/>
+    <row r="848" ht="15.75" customHeight="1"/>
+    <row r="849" ht="15.75" customHeight="1"/>
+    <row r="850" ht="15.75" customHeight="1"/>
+    <row r="851" ht="15.75" customHeight="1"/>
+    <row r="852" ht="15.75" customHeight="1"/>
+    <row r="853" ht="15.75" customHeight="1"/>
+    <row r="854" ht="15.75" customHeight="1"/>
+    <row r="855" ht="15.75" customHeight="1"/>
+    <row r="856" ht="15.75" customHeight="1"/>
+    <row r="857" ht="15.75" customHeight="1"/>
+    <row r="858" ht="15.75" customHeight="1"/>
+    <row r="859" ht="15.75" customHeight="1"/>
+    <row r="860" ht="15.75" customHeight="1"/>
+    <row r="861" ht="15.75" customHeight="1"/>
+    <row r="862" ht="15.75" customHeight="1"/>
+    <row r="863" ht="15.75" customHeight="1"/>
+    <row r="864" ht="15.75" customHeight="1"/>
+    <row r="865" ht="15.75" customHeight="1"/>
+    <row r="866" ht="15.75" customHeight="1"/>
+    <row r="867" ht="15.75" customHeight="1"/>
+    <row r="868" ht="15.75" customHeight="1"/>
+    <row r="869" ht="15.75" customHeight="1"/>
+    <row r="870" ht="15.75" customHeight="1"/>
+    <row r="871" ht="15.75" customHeight="1"/>
+    <row r="872" ht="15.75" customHeight="1"/>
+    <row r="873" ht="15.75" customHeight="1"/>
+    <row r="874" ht="15.75" customHeight="1"/>
+    <row r="875" ht="15.75" customHeight="1"/>
+    <row r="876" ht="15.75" customHeight="1"/>
+    <row r="877" ht="15.75" customHeight="1"/>
+    <row r="878" ht="15.75" customHeight="1"/>
+    <row r="879" ht="15.75" customHeight="1"/>
+    <row r="880" ht="15.75" customHeight="1"/>
+    <row r="881" ht="15.75" customHeight="1"/>
+    <row r="882" ht="15.75" customHeight="1"/>
+    <row r="883" ht="15.75" customHeight="1"/>
+    <row r="884" ht="15.75" customHeight="1"/>
+    <row r="885" ht="15.75" customHeight="1"/>
+    <row r="886" ht="15.75" customHeight="1"/>
+    <row r="887" ht="15.75" customHeight="1"/>
+    <row r="888" ht="15.75" customHeight="1"/>
+    <row r="889" ht="15.75" customHeight="1"/>
+    <row r="890" ht="15.75" customHeight="1"/>
+    <row r="891" ht="15.75" customHeight="1"/>
+    <row r="892" ht="15.75" customHeight="1"/>
+    <row r="893" ht="15.75" customHeight="1"/>
+    <row r="894" ht="15.75" customHeight="1"/>
+    <row r="895" ht="15.75" customHeight="1"/>
+    <row r="896" ht="15.75" customHeight="1"/>
+    <row r="897" ht="15.75" customHeight="1"/>
+    <row r="898" ht="15.75" customHeight="1"/>
+    <row r="899" ht="15.75" customHeight="1"/>
+    <row r="900" ht="15.75" customHeight="1"/>
+    <row r="901" ht="15.75" customHeight="1"/>
+    <row r="902" ht="15.75" customHeight="1"/>
+    <row r="903" ht="15.75" customHeight="1"/>
+    <row r="904" ht="15.75" customHeight="1"/>
+    <row r="905" ht="15.75" customHeight="1"/>
+    <row r="906" ht="15.75" customHeight="1"/>
+    <row r="907" ht="15.75" customHeight="1"/>
+    <row r="908" ht="15.75" customHeight="1"/>
+    <row r="909" ht="15.75" customHeight="1"/>
+    <row r="910" ht="15.75" customHeight="1"/>
+    <row r="911" ht="15.75" customHeight="1"/>
+    <row r="912" ht="15.75" customHeight="1"/>
+    <row r="913" ht="15.75" customHeight="1"/>
+    <row r="914" ht="15.75" customHeight="1"/>
+    <row r="915" ht="15.75" customHeight="1"/>
+    <row r="916" ht="15.75" customHeight="1"/>
+    <row r="917" ht="15.75" customHeight="1"/>
+    <row r="918" ht="15.75" customHeight="1"/>
+    <row r="919" ht="15.75" customHeight="1"/>
+    <row r="920" ht="15.75" customHeight="1"/>
+    <row r="921" ht="15.75" customHeight="1"/>
+    <row r="922" ht="15.75" customHeight="1"/>
+    <row r="923" ht="15.75" customHeight="1"/>
+    <row r="924" ht="15.75" customHeight="1"/>
+    <row r="925" ht="15.75" customHeight="1"/>
+    <row r="926" ht="15.75" customHeight="1"/>
+    <row r="927" ht="15.75" customHeight="1"/>
+    <row r="928" ht="15.75" customHeight="1"/>
+    <row r="929" ht="15.75" customHeight="1"/>
+    <row r="930" ht="15.75" customHeight="1"/>
+    <row r="931" ht="15.75" customHeight="1"/>
+    <row r="932" ht="15.75" customHeight="1"/>
+    <row r="933" ht="15.75" customHeight="1"/>
+    <row r="934" ht="15.75" customHeight="1"/>
+    <row r="935" ht="15.75" customHeight="1"/>
+    <row r="936" ht="15.75" customHeight="1"/>
+    <row r="937" ht="15.75" customHeight="1"/>
+    <row r="938" ht="15.75" customHeight="1"/>
+    <row r="939" ht="15.75" customHeight="1"/>
+    <row r="940" ht="15.75" customHeight="1"/>
+    <row r="941" ht="15.75" customHeight="1"/>
+    <row r="942" ht="15.75" customHeight="1"/>
+    <row r="943" ht="15.75" customHeight="1"/>
+    <row r="944" ht="15.75" customHeight="1"/>
+    <row r="945" ht="15.75" customHeight="1"/>
+    <row r="946" ht="15.75" customHeight="1"/>
+    <row r="947" ht="15.75" customHeight="1"/>
+    <row r="948" ht="15.75" customHeight="1"/>
+    <row r="949" ht="15.75" customHeight="1"/>
+    <row r="950" ht="15.75" customHeight="1"/>
+    <row r="951" ht="15.75" customHeight="1"/>
+    <row r="952" ht="15.75" customHeight="1"/>
+    <row r="953" ht="15.75" customHeight="1"/>
+    <row r="954" ht="15.75" customHeight="1"/>
+    <row r="955" ht="15.75" customHeight="1"/>
+    <row r="956" ht="15.75" customHeight="1"/>
+    <row r="957" ht="15.75" customHeight="1"/>
+    <row r="958" ht="15.75" customHeight="1"/>
+    <row r="959" ht="15.75" customHeight="1"/>
+    <row r="960" ht="15.75" customHeight="1"/>
+    <row r="961" ht="15.75" customHeight="1"/>
+    <row r="962" ht="15.75" customHeight="1"/>
+    <row r="963" ht="15.75" customHeight="1"/>
+    <row r="964" ht="15.75" customHeight="1"/>
+    <row r="965" ht="15.75" customHeight="1"/>
+    <row r="966" ht="15.75" customHeight="1"/>
+    <row r="967" ht="15.75" customHeight="1"/>
+    <row r="968" ht="15.75" customHeight="1"/>
+    <row r="969" ht="15.75" customHeight="1"/>
+    <row r="970" ht="15.75" customHeight="1"/>
+    <row r="971" ht="15.75" customHeight="1"/>
+    <row r="972" ht="15.75" customHeight="1"/>
+    <row r="973" ht="15.75" customHeight="1"/>
+    <row r="974" ht="15.75" customHeight="1"/>
+    <row r="975" ht="15.75" customHeight="1"/>
+    <row r="976" ht="15.75" customHeight="1"/>
+    <row r="977" ht="15.75" customHeight="1"/>
+    <row r="978" ht="15.75" customHeight="1"/>
+    <row r="979" ht="15.75" customHeight="1"/>
+    <row r="980" ht="15.75" customHeight="1"/>
+    <row r="981" ht="15.75" customHeight="1"/>
+    <row r="982" ht="15.75" customHeight="1"/>
+    <row r="983" ht="15.75" customHeight="1"/>
+    <row r="984" ht="15.75" customHeight="1"/>
+    <row r="985" ht="15.75" customHeight="1"/>
+    <row r="986" ht="15.75" customHeight="1"/>
+    <row r="987" ht="15.75" customHeight="1"/>
+    <row r="988" ht="15.75" customHeight="1"/>
+    <row r="989" ht="15.75" customHeight="1"/>
+    <row r="990" ht="15.75" customHeight="1"/>
+    <row r="991" ht="15.75" customHeight="1"/>
+    <row r="992" ht="15.75" customHeight="1"/>
+    <row r="993" ht="15.75" customHeight="1"/>
+    <row r="994" ht="15.75" customHeight="1"/>
+    <row r="995" ht="15.75" customHeight="1"/>
+    <row r="996" ht="15.75" customHeight="1"/>
+    <row r="997" ht="15.75" customHeight="1"/>
+    <row r="998" ht="15.75" customHeight="1"/>
+    <row r="999" ht="15.75" customHeight="1"/>
+    <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="A1:A3"/>
@@ -3774,7 +3785,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>3</v>
@@ -6206,7 +6217,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>4</v>
@@ -6216,7 +6227,7 @@
       <c r="A2" s="1">
         <v>0.0</v>
       </c>
-      <c r="B2" s="3">
+      <c r="B2" s="4">
         <v>1.0</v>
       </c>
     </row>
@@ -6224,7 +6235,7 @@
       <c r="A3" s="1">
         <v>1.0</v>
       </c>
-      <c r="B3" s="3">
+      <c r="B3" s="4">
         <v>1.1</v>
       </c>
     </row>
@@ -6232,7 +6243,7 @@
       <c r="A4" s="1">
         <v>2.0</v>
       </c>
-      <c r="B4" s="3">
+      <c r="B4" s="4">
         <v>1.2</v>
       </c>
     </row>
@@ -6240,7 +6251,7 @@
       <c r="A5" s="1">
         <v>3.0</v>
       </c>
-      <c r="B5" s="3">
+      <c r="B5" s="4">
         <v>1.3</v>
       </c>
     </row>
@@ -6248,7 +6259,7 @@
       <c r="A6" s="1">
         <v>4.0</v>
       </c>
-      <c r="B6" s="3">
+      <c r="B6" s="4">
         <v>1.4</v>
       </c>
     </row>
@@ -6256,7 +6267,7 @@
       <c r="A7" s="1">
         <v>5.0</v>
       </c>
-      <c r="B7" s="3">
+      <c r="B7" s="4">
         <v>1.5</v>
       </c>
     </row>
@@ -6264,7 +6275,7 @@
       <c r="A8" s="1">
         <v>6.0</v>
       </c>
-      <c r="B8" s="3">
+      <c r="B8" s="4">
         <v>1.6</v>
       </c>
     </row>
@@ -6272,7 +6283,7 @@
       <c r="A9" s="1">
         <v>7.0</v>
       </c>
-      <c r="B9" s="3">
+      <c r="B9" s="4">
         <v>1.7</v>
       </c>
     </row>
@@ -6280,7 +6291,7 @@
       <c r="A10" s="1">
         <v>8.0</v>
       </c>
-      <c r="B10" s="3">
+      <c r="B10" s="4">
         <v>1.8</v>
       </c>
     </row>
@@ -6288,7 +6299,7 @@
       <c r="A11" s="1">
         <v>9.0</v>
       </c>
-      <c r="B11" s="3">
+      <c r="B11" s="4">
         <v>1.9</v>
       </c>
     </row>
@@ -6296,7 +6307,7 @@
       <c r="A12" s="1">
         <v>10.0</v>
       </c>
-      <c r="B12" s="3">
+      <c r="B12" s="4">
         <v>2.0</v>
       </c>
     </row>
@@ -6304,7 +6315,7 @@
       <c r="A13" s="1">
         <v>11.0</v>
       </c>
-      <c r="B13" s="3">
+      <c r="B13" s="4">
         <v>2.1</v>
       </c>
     </row>
@@ -6312,7 +6323,7 @@
       <c r="A14" s="1">
         <v>12.0</v>
       </c>
-      <c r="B14" s="3">
+      <c r="B14" s="4">
         <v>2.2</v>
       </c>
     </row>
@@ -6320,7 +6331,7 @@
       <c r="A15" s="1">
         <v>13.0</v>
       </c>
-      <c r="B15" s="3">
+      <c r="B15" s="4">
         <v>2.3</v>
       </c>
     </row>
@@ -6328,7 +6339,7 @@
       <c r="A16" s="1">
         <v>14.0</v>
       </c>
-      <c r="B16" s="3">
+      <c r="B16" s="4">
         <v>2.3</v>
       </c>
     </row>
@@ -6336,7 +6347,7 @@
       <c r="A17" s="1">
         <v>15.0</v>
       </c>
-      <c r="B17" s="3">
+      <c r="B17" s="4">
         <v>2.4</v>
       </c>
     </row>
@@ -6344,7 +6355,7 @@
       <c r="A18" s="1">
         <v>16.0</v>
       </c>
-      <c r="B18" s="3">
+      <c r="B18" s="4">
         <v>2.5</v>
       </c>
     </row>
@@ -6352,7 +6363,7 @@
       <c r="A19" s="1">
         <v>17.0</v>
       </c>
-      <c r="B19" s="3">
+      <c r="B19" s="4">
         <v>2.6</v>
       </c>
     </row>
@@ -6360,7 +6371,7 @@
       <c r="A20" s="1">
         <v>18.0</v>
       </c>
-      <c r="B20" s="3">
+      <c r="B20" s="4">
         <v>2.7</v>
       </c>
     </row>
@@ -6368,7 +6379,7 @@
       <c r="A21" s="1">
         <v>19.0</v>
       </c>
-      <c r="B21" s="3">
+      <c r="B21" s="4">
         <v>2.8</v>
       </c>
     </row>
@@ -6376,7 +6387,7 @@
       <c r="A22" s="1">
         <v>20.0</v>
       </c>
-      <c r="B22" s="3">
+      <c r="B22" s="4">
         <v>2.9</v>
       </c>
     </row>
@@ -6384,7 +6395,7 @@
       <c r="A23" s="1">
         <v>21.0</v>
       </c>
-      <c r="B23" s="3">
+      <c r="B23" s="4">
         <v>3.0</v>
       </c>
     </row>
@@ -6392,7 +6403,7 @@
       <c r="A24" s="1">
         <v>22.0</v>
       </c>
-      <c r="B24" s="3">
+      <c r="B24" s="4">
         <v>3.1</v>
       </c>
     </row>
@@ -6400,7 +6411,7 @@
       <c r="A25" s="1">
         <v>23.0</v>
       </c>
-      <c r="B25" s="3">
+      <c r="B25" s="4">
         <v>3.2</v>
       </c>
     </row>
@@ -6408,7 +6419,7 @@
       <c r="A26" s="1">
         <v>24.0</v>
       </c>
-      <c r="B26" s="3">
+      <c r="B26" s="4">
         <v>3.3</v>
       </c>
     </row>
@@ -6416,7 +6427,7 @@
       <c r="A27" s="1">
         <v>25.0</v>
       </c>
-      <c r="B27" s="3">
+      <c r="B27" s="4">
         <v>3.4</v>
       </c>
     </row>
@@ -6424,7 +6435,7 @@
       <c r="A28" s="1">
         <v>26.0</v>
       </c>
-      <c r="B28" s="3">
+      <c r="B28" s="4">
         <v>3.5</v>
       </c>
     </row>
@@ -6432,7 +6443,7 @@
       <c r="A29" s="1">
         <v>27.0</v>
       </c>
-      <c r="B29" s="3">
+      <c r="B29" s="4">
         <v>3.6</v>
       </c>
     </row>
@@ -6440,7 +6451,7 @@
       <c r="A30" s="1">
         <v>28.0</v>
       </c>
-      <c r="B30" s="3">
+      <c r="B30" s="4">
         <v>3.7</v>
       </c>
     </row>
@@ -6448,7 +6459,7 @@
       <c r="A31" s="1">
         <v>29.0</v>
       </c>
-      <c r="B31" s="3">
+      <c r="B31" s="4">
         <v>3.8</v>
       </c>
     </row>
@@ -6456,7 +6467,7 @@
       <c r="A32" s="1">
         <v>30.0</v>
       </c>
-      <c r="B32" s="3">
+      <c r="B32" s="4">
         <v>3.9</v>
       </c>
     </row>
@@ -6464,7 +6475,7 @@
       <c r="A33" s="1">
         <v>31.0</v>
       </c>
-      <c r="B33" s="3">
+      <c r="B33" s="4">
         <v>4.0</v>
       </c>
     </row>
@@ -6472,7 +6483,7 @@
       <c r="A34" s="1">
         <v>32.0</v>
       </c>
-      <c r="B34" s="3">
+      <c r="B34" s="4">
         <v>4.1</v>
       </c>
     </row>
@@ -6480,7 +6491,7 @@
       <c r="A35" s="1">
         <v>33.0</v>
       </c>
-      <c r="B35" s="3">
+      <c r="B35" s="4">
         <v>4.3</v>
       </c>
     </row>
@@ -6488,7 +6499,7 @@
       <c r="A36" s="1">
         <v>34.0</v>
       </c>
-      <c r="B36" s="3">
+      <c r="B36" s="4">
         <v>4.4</v>
       </c>
     </row>
@@ -6496,7 +6507,7 @@
       <c r="A37" s="1">
         <v>35.0</v>
       </c>
-      <c r="B37" s="3">
+      <c r="B37" s="4">
         <v>4.5</v>
       </c>
     </row>
@@ -6504,7 +6515,7 @@
       <c r="A38" s="1">
         <v>36.0</v>
       </c>
-      <c r="B38" s="3">
+      <c r="B38" s="4">
         <v>4.7</v>
       </c>
     </row>
@@ -6512,7 +6523,7 @@
       <c r="A39" s="1">
         <v>37.0</v>
       </c>
-      <c r="B39" s="3">
+      <c r="B39" s="4">
         <v>4.8</v>
       </c>
     </row>
@@ -6520,7 +6531,7 @@
       <c r="A40" s="1">
         <v>38.0</v>
       </c>
-      <c r="B40" s="3">
+      <c r="B40" s="4">
         <v>5.0</v>
       </c>
     </row>
@@ -6528,7 +6539,7 @@
       <c r="A41" s="1">
         <v>39.0</v>
       </c>
-      <c r="B41" s="3">
+      <c r="B41" s="4">
         <v>5.1</v>
       </c>
     </row>
@@ -6536,7 +6547,7 @@
       <c r="A42" s="1">
         <v>40.0</v>
       </c>
-      <c r="B42" s="3">
+      <c r="B42" s="4">
         <v>5.3</v>
       </c>
     </row>
@@ -6544,7 +6555,7 @@
       <c r="A43" s="1">
         <v>41.0</v>
       </c>
-      <c r="B43" s="3">
+      <c r="B43" s="4">
         <v>5.4</v>
       </c>
     </row>
@@ -6552,7 +6563,7 @@
       <c r="A44" s="1">
         <v>42.0</v>
       </c>
-      <c r="B44" s="3">
+      <c r="B44" s="4">
         <v>5.6</v>
       </c>
     </row>
@@ -6560,7 +6571,7 @@
       <c r="A45" s="1">
         <v>43.0</v>
       </c>
-      <c r="B45" s="3">
+      <c r="B45" s="4">
         <v>5.7</v>
       </c>
     </row>
@@ -6568,7 +6579,7 @@
       <c r="A46" s="1">
         <v>44.0</v>
       </c>
-      <c r="B46" s="3">
+      <c r="B46" s="4">
         <v>5.8</v>
       </c>
     </row>
@@ -6576,7 +6587,7 @@
       <c r="A47" s="1">
         <v>45.0</v>
       </c>
-      <c r="B47" s="3">
+      <c r="B47" s="4">
         <v>6.0</v>
       </c>
     </row>
@@ -6584,7 +6595,7 @@
       <c r="A48" s="1">
         <v>46.0</v>
       </c>
-      <c r="B48" s="3">
+      <c r="B48" s="4">
         <v>6.1</v>
       </c>
     </row>
@@ -6592,7 +6603,7 @@
       <c r="A49" s="1">
         <v>47.0</v>
       </c>
-      <c r="B49" s="3">
+      <c r="B49" s="4">
         <v>6.3</v>
       </c>
     </row>
@@ -6600,7 +6611,7 @@
       <c r="A50" s="1">
         <v>48.0</v>
       </c>
-      <c r="B50" s="3">
+      <c r="B50" s="4">
         <v>6.4</v>
       </c>
     </row>
@@ -6608,7 +6619,7 @@
       <c r="A51" s="1">
         <v>49.0</v>
       </c>
-      <c r="B51" s="3">
+      <c r="B51" s="4">
         <v>6.6</v>
       </c>
     </row>
@@ -6616,7 +6627,7 @@
       <c r="A52" s="1">
         <v>50.0</v>
       </c>
-      <c r="B52" s="3">
+      <c r="B52" s="4">
         <v>6.7</v>
       </c>
     </row>
@@ -6624,7 +6635,7 @@
       <c r="A53" s="1">
         <v>51.0</v>
       </c>
-      <c r="B53" s="3">
+      <c r="B53" s="4">
         <v>6.9</v>
       </c>
     </row>
@@ -6632,7 +6643,7 @@
       <c r="A54" s="1">
         <v>52.0</v>
       </c>
-      <c r="B54" s="3">
+      <c r="B54" s="4">
         <v>7.0</v>
       </c>
     </row>
@@ -7602,7 +7613,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>3</v>
@@ -8017,10 +8028,10 @@
       </c>
     </row>
     <row r="53" ht="15.75" customHeight="1">
-      <c r="B53" s="3"/>
+      <c r="B53" s="4"/>
     </row>
     <row r="54" ht="15.75" customHeight="1">
-      <c r="B54" s="3"/>
+      <c r="B54" s="4"/>
     </row>
     <row r="55" ht="15.75" customHeight="1"/>
     <row r="56" ht="15.75" customHeight="1"/>
@@ -8988,10 +8999,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="38" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="B1" s="39" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C1" s="40"/>
       <c r="D1" s="40"/>
@@ -9000,21 +9011,21 @@
     <row r="2">
       <c r="A2" s="42"/>
       <c r="B2" s="43" t="s">
-        <v>24</v>
+        <v>59</v>
       </c>
       <c r="C2" s="44" t="s">
-        <v>27</v>
+        <v>60</v>
       </c>
       <c r="D2" s="44" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="E2" s="45" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="46" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="B3" s="47">
         <v>4.0</v>

</xml_diff>